<commit_message>
Add execution alerts and refine dark theme and validation
</commit_message>
<xml_diff>
--- a/Modelo-SGP.xlsx
+++ b/Modelo-SGP.xlsx
@@ -6153,10 +6153,12 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:D78"/>
   <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="110.83203125" customWidth="1"/>
+    <col min="1" max="1" width="34.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="95.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6166,151 +6168,925 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Datas</v>
+        <v>Como preencher</v>
       </c>
       <c r="B2" t="str">
-        <v>AAAA-MM-DD como texto, ou células de data do Excel.</v>
+        <v>Use uma linha por registro. Não altere os nomes das abas nem os cabeçalhos. Campos com * são obrigatórios. Datas preferencialmente em AAAA-MM-DD.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>IDs</v>
+        <v>Legenda</v>
       </c>
       <c r="B3" t="str">
-        <v>IDs únicos em Demandas e Pessoas; referências exatas nas outras abas. Não renomeie IDs em apenas uma aba.</v>
+        <v>Exemplo mostra o tipo de valor esperado; listas devem usar exatamente uma das opções indicadas.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Importação</v>
+        <v>Datas</v>
       </c>
       <c r="B4" t="str">
-        <v>Substitui toda a base somente depois da pré-validação e confirmação. Abas vazias são permitidas com cabeçalhos.</v>
+        <v>AAAA-MM-DD como texto, ou células de data do Excel.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Frentes</v>
+        <v>IDs</v>
       </c>
       <c r="B5" t="str">
-        <v>Produção; Qualidade; Torque; Automação Industrial; Inovação IoT</v>
+        <v>IDs únicos em Demandas e Pessoas; referências exatas nas outras abas. Não renomeie IDs em apenas uma aba.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Status</v>
+        <v>Importação</v>
       </c>
       <c r="B6" t="str">
-        <v>Não iniciado; Em andamento; Aguardando cliente; Aguardando aprovação; Bloqueado; Em risco; Concluído; Cancelado</v>
+        <v>Substitui toda a base somente depois da pré-validação e confirmação. Abas vazias são permitidas com cabeçalhos.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Fases</v>
+        <v>Frentes</v>
       </c>
       <c r="B7" t="str">
-        <v>Entrada; Levantamento; Proposta; Aprovação; Planejamento; Desenvolvimento; Homologação; Implantação; Fechamento; Concluído; Aguardando Cliente</v>
+        <v>Produção; Qualidade; Torque; Automação Industrial; Inovação IoT</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Risco</v>
+        <v>Status</v>
       </c>
       <c r="B8" t="str">
-        <v>Nenhum; Baixa; Média; Alta; Crítica</v>
+        <v>Não iniciado; Em andamento; Aguardando cliente; Aguardando aprovação; Bloqueado; Em risco; Concluído; Cancelado</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Tipo</v>
+        <v>Fases</v>
       </c>
       <c r="B9" t="str">
-        <v>Projeto; Proposta; Melhoria; Evolução; Ticket N3; Outro</v>
+        <v>Entrada; Levantamento; Proposta; Aprovação; Planejamento; Desenvolvimento; Homologação; Implantação; Fechamento; Concluído; Aguardando Cliente</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Função</v>
+        <v>Risco</v>
       </c>
       <c r="B10" t="str">
-        <v>Tech Leader; Analista; Desenvolvedor; PMO; Plan; Business Operations; Outro</v>
+        <v>Nenhum; Baixa; Média; Alta; Crítica</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Ativo</v>
+        <v>Tipo</v>
       </c>
       <c r="B11" t="str">
-        <v>Sim; Não</v>
+        <v>Projeto; Proposta; Melhoria; Evolução; Ticket N3; Outro</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Capacidade</v>
+        <v>Função</v>
       </c>
       <c r="B12" t="str">
-        <v>Capacidade mensal em horas, proporcional aos dias corridos do mês. Horas alocadas são totais do intervalo, distribuídas uniformemente pelos dias corridos. Feriados não são descontados. Percentual é informativo; Horas alimenta a capacidade.</v>
+        <v>Tech Leader; Analista; Desenvolvedor; PMO; Plan; Business Operations; Outro</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Marcos</v>
+        <v>Ativo</v>
       </c>
       <c r="B13" t="str">
-        <v>Marcos cadastrados prevalecem sobre datas equivalentes da demanda. Entrega técnica e final são também consideradas quando não houver marco equivalente.</v>
+        <v>Sim; Não</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Segurança</v>
+        <v>Capacidade</v>
       </c>
       <c r="B14" t="str">
-        <v>Somente dados fictícios neste modelo. Cópias Excel são sua responsabilidade; armazenamento local não sincroniza computadores.</v>
+        <v>Capacidade mensal em horas, proporcional aos dias corridos do mês. Horas alocadas são totais do intervalo, distribuídas uniformemente pelos dias corridos. Feriados não são descontados. Percentual é informativo; Horas alimenta a capacidade.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Demandas — obrigatórios</v>
+        <v>Marcos</v>
       </c>
       <c r="B15" t="str">
-        <v>ID; Código; Nome da Demanda; Tipo; Frente; Fase Atual; Status; Data Início; Data Final Prevista</v>
+        <v>Marcos cadastrados prevalecem sobre datas equivalentes da demanda. Entrega técnica e final são também consideradas quando não houver marco equivalente.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Pessoas — obrigatórios</v>
+        <v>Segurança</v>
       </c>
       <c r="B16" t="str">
-        <v>ID; Nome; Função; Frente Principal; Capacidade Mensal; Ativo</v>
+        <v>Somente dados fictícios neste modelo. Cópias Excel são sua responsabilidade; armazenamento local não sincroniza computadores.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Alocacoes — obrigatórios</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Pessoa ID; Demanda ID; Data Início; Data Fim; Horas</v>
+        <f>Campo</f>
+        <v>Demandas — instruções por coluna</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Fases — obrigatórios</v>
+        <v>ID</v>
       </c>
       <c r="B18" t="str">
-        <v>Demanda ID; Fase; Data Início; Data Fim; Status</v>
+        <v>id</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D18" t="str">
+        <v>ID único; não duplique e mantenha as referências nas outras abas.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
+        <v>Código</v>
+      </c>
+      <c r="B19" t="str">
+        <v>code</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Código curto e único da demanda (ex.: P001).</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Nome da Demanda</v>
+      </c>
+      <c r="B20" t="str">
+        <v>name</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Texto para Nome da Demanda; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Descrição resumida</v>
+      </c>
+      <c r="B21" t="str">
+        <v>description</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Texto para Descrição resumida; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Tipo</v>
+      </c>
+      <c r="B22" t="str">
+        <v>type</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Use Projeto, Proposta, Melhoria, Evolução, Ticket N3 ou Outro.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Frente</v>
+      </c>
+      <c r="B23" t="str">
+        <v>front</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Use uma frente válida da lista na aba LEIA-ME.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Plan</v>
+      </c>
+      <c r="B24" t="str">
+        <v>plan</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Texto para Plan; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>PMO</v>
+      </c>
+      <c r="B25" t="str">
+        <v>pmo</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Texto para PMO; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Tech Leader</v>
+      </c>
+      <c r="B26" t="str">
+        <v>leader</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Texto para Tech Leader; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Responsável BO</v>
+      </c>
+      <c r="B27" t="str">
+        <v>bo</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Texto para Responsável BO; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Fase Atual</v>
+      </c>
+      <c r="B28" t="str">
+        <v>phase</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Use uma fase válida da lista na aba LEIA-ME.</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Status</v>
+      </c>
+      <c r="B29" t="str">
+        <v>status</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Use um status válido da lista na aba LEIA-ME.</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Data de Entrada</v>
+      </c>
+      <c r="B30" t="str">
+        <v>entry</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Data Início</v>
+      </c>
+      <c r="B31" t="str">
+        <v>start</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Data Entrega Técnica</v>
+      </c>
+      <c r="B32" t="str">
+        <v>technical</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Data Homologação</v>
+      </c>
+      <c r="B33" t="str">
+        <v>homologation</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Data Implantação</v>
+      </c>
+      <c r="B34" t="str">
+        <v>deployment</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Data Final Prevista</v>
+      </c>
+      <c r="B35" t="str">
+        <v>end</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Horas Estimadas</v>
+      </c>
+      <c r="B36" t="str">
+        <v>estimated</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Número não negativo (ex.: 160).</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Horas Consumidas</v>
+      </c>
+      <c r="B37" t="str">
+        <v>consumed</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Número não negativo (ex.: 160).</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Percentual de Conclusão</v>
+      </c>
+      <c r="B38" t="str">
+        <v>progress</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Percentual de 0 a 100 (ex.: 75).</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Próximo Marco</v>
+      </c>
+      <c r="B39" t="str">
+        <v>next</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Texto para Próximo Marco; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Data Próximo Marco</v>
+      </c>
+      <c r="B40" t="str">
+        <v>nextDate</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Dependência</v>
+      </c>
+      <c r="B41" t="str">
+        <v>dependency</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Texto para Dependência; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Responsável pela Dependência</v>
+      </c>
+      <c r="B42" t="str">
+        <v>dependencyOwner</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Texto para Responsável pela Dependência; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Risco</v>
+      </c>
+      <c r="B43" t="str">
+        <v>risk</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Use Nenhum, Baixa, Média, Alta ou Crítica.</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Descrição do Risco</v>
+      </c>
+      <c r="B44" t="str">
+        <v>riskDescription</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Texto para Descrição do Risco; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Link Git</v>
+      </c>
+      <c r="B45" t="str">
+        <v>git</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Texto para Link Git; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Observação</v>
+      </c>
+      <c r="B46" t="str">
+        <v>notes</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Texto para Observação; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <f>Campo</f>
+        <v>Pessoas — instruções por coluna</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B48" t="str">
+        <v>id</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D48" t="str">
+        <v>ID único; não duplique e mantenha as referências nas outras abas.</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Nome</v>
+      </c>
+      <c r="B49" t="str">
+        <v>name</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Texto para Nome; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Função</v>
+      </c>
+      <c r="B50" t="str">
+        <v>role</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Texto para Função; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Frente Principal</v>
+      </c>
+      <c r="B51" t="str">
+        <v>front</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Use uma frente válida da lista na aba LEIA-ME.</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Tech Leader</v>
+      </c>
+      <c r="B52" t="str">
+        <v>leader</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Texto para Tech Leader; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Capacidade Mensal</v>
+      </c>
+      <c r="B53" t="str">
+        <v>capacity</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Capacidade mensal em horas; número não negativo.</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Ativo</v>
+      </c>
+      <c r="B54" t="str">
+        <v>active</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Use Sim ou Não.</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <f>Campo</f>
+        <v>Alocacoes — instruções por coluna</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Pessoa ID</v>
+      </c>
+      <c r="B56" t="str">
+        <v>person</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D56" t="str">
+        <v>ID da pessoa existente.</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Demanda ID</v>
+      </c>
+      <c r="B57" t="str">
+        <v>demand</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D57" t="str">
+        <v>ID da demanda existente.</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Data Início</v>
+      </c>
+      <c r="B58" t="str">
+        <v>start</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Data Fim</v>
+      </c>
+      <c r="B59" t="str">
+        <v>end</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Horas</v>
+      </c>
+      <c r="B60" t="str">
+        <v>hours</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Horas totais do intervalo; número não negativo.</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Percentual</v>
+      </c>
+      <c r="B61" t="str">
+        <v>percent</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Percentual informativo de 0 a 100.</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <f>Campo</f>
+        <v>Fases — instruções por coluna</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>Demanda ID</v>
+      </c>
+      <c r="B63" t="str">
+        <v>demand</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D63" t="str">
+        <v>ID da demanda existente.</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Fase</v>
+      </c>
+      <c r="B64" t="str">
+        <v>phase</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Use uma fase válida da lista na aba LEIA-ME.</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>Data Início</v>
+      </c>
+      <c r="B65" t="str">
+        <v>start</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Data Fim</v>
+      </c>
+      <c r="B66" t="str">
+        <v>end</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Status</v>
+      </c>
+      <c r="B67" t="str">
+        <v>status</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Use um status válido da lista na aba LEIA-ME.</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <f>Campo</f>
+        <v>Marcos — instruções por coluna</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>Demanda ID</v>
+      </c>
+      <c r="B69" t="str">
+        <v>demand</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D69" t="str">
+        <v>ID da demanda existente.</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Marco</v>
+      </c>
+      <c r="B70" t="str">
+        <v>name</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Texto para Marco; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Data</v>
+      </c>
+      <c r="B71" t="str">
+        <v>date</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Status</v>
+      </c>
+      <c r="B72" t="str">
+        <v>status</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Use um status válido da lista na aba LEIA-ME.</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Observação</v>
+      </c>
+      <c r="B73" t="str">
+        <v>notes</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Texto para Observação; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>Demandas — obrigatórios</v>
+      </c>
+      <c r="B74" t="str">
+        <v>ID; Código; Nome da Demanda; Tipo; Frente; Fase Atual; Status; Data Início; Data Final Prevista</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>Pessoas — obrigatórios</v>
+      </c>
+      <c r="B75" t="str">
+        <v>ID; Nome; Função; Frente Principal; Capacidade Mensal; Ativo</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>Alocacoes — obrigatórios</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Pessoa ID; Demanda ID; Data Início; Data Fim; Horas</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>Fases — obrigatórios</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Demanda ID; Fase; Data Início; Data Fim; Status</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
         <v>Marcos — obrigatórios</v>
       </c>
-      <c r="B19" t="str">
+      <c r="B78" t="str">
         <v>Demanda ID; Marco; Data; Status</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D78"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Calculate allocation percentages automatically
</commit_message>
<xml_diff>
--- a/Modelo-SGP.xlsx
+++ b/Modelo-SGP.xlsx
@@ -2472,8 +2472,8 @@
       <c r="E2">
         <v>38</v>
       </c>
-      <c r="F2" t="str">
-        <v/>
+      <c r="F2">
+        <v>23.75</v>
       </c>
     </row>
     <row r="3">
@@ -2492,8 +2492,8 @@
       <c r="E3">
         <v>40</v>
       </c>
-      <c r="F3" t="str">
-        <v/>
+      <c r="F3">
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -2512,8 +2512,8 @@
       <c r="E4">
         <v>42</v>
       </c>
-      <c r="F4" t="str">
-        <v/>
+      <c r="F4">
+        <v>26.25</v>
       </c>
     </row>
     <row r="5">
@@ -2532,8 +2532,8 @@
       <c r="E5">
         <v>44</v>
       </c>
-      <c r="F5" t="str">
-        <v/>
+      <c r="F5">
+        <v>27.500000000000004</v>
       </c>
     </row>
     <row r="6">
@@ -2552,8 +2552,8 @@
       <c r="E6">
         <v>42</v>
       </c>
-      <c r="F6" t="str">
-        <v/>
+      <c r="F6">
+        <v>26.25</v>
       </c>
     </row>
     <row r="7">
@@ -2572,8 +2572,8 @@
       <c r="E7">
         <v>44</v>
       </c>
-      <c r="F7" t="str">
-        <v/>
+      <c r="F7">
+        <v>27.500000000000004</v>
       </c>
     </row>
     <row r="8">
@@ -2592,8 +2592,8 @@
       <c r="E8">
         <v>46</v>
       </c>
-      <c r="F8" t="str">
-        <v/>
+      <c r="F8">
+        <v>28.749999999999996</v>
       </c>
     </row>
     <row r="9">
@@ -2612,8 +2612,8 @@
       <c r="E9">
         <v>48</v>
       </c>
-      <c r="F9" t="str">
-        <v/>
+      <c r="F9">
+        <v>30</v>
       </c>
     </row>
     <row r="10">
@@ -2632,8 +2632,8 @@
       <c r="E10">
         <v>46</v>
       </c>
-      <c r="F10" t="str">
-        <v/>
+      <c r="F10">
+        <v>28.749999999999996</v>
       </c>
     </row>
     <row r="11">
@@ -2652,8 +2652,8 @@
       <c r="E11">
         <v>48</v>
       </c>
-      <c r="F11" t="str">
-        <v/>
+      <c r="F11">
+        <v>30</v>
       </c>
     </row>
     <row r="12">
@@ -2672,8 +2672,8 @@
       <c r="E12">
         <v>50</v>
       </c>
-      <c r="F12" t="str">
-        <v/>
+      <c r="F12">
+        <v>31.25</v>
       </c>
     </row>
     <row r="13">
@@ -2692,8 +2692,8 @@
       <c r="E13">
         <v>52</v>
       </c>
-      <c r="F13" t="str">
-        <v/>
+      <c r="F13">
+        <v>32.5</v>
       </c>
     </row>
     <row r="14">
@@ -2712,8 +2712,8 @@
       <c r="E14">
         <v>38</v>
       </c>
-      <c r="F14" t="str">
-        <v/>
+      <c r="F14">
+        <v>23.75</v>
       </c>
     </row>
     <row r="15">
@@ -2732,8 +2732,8 @@
       <c r="E15">
         <v>40</v>
       </c>
-      <c r="F15" t="str">
-        <v/>
+      <c r="F15">
+        <v>25</v>
       </c>
     </row>
     <row r="16">
@@ -2752,8 +2752,8 @@
       <c r="E16">
         <v>42</v>
       </c>
-      <c r="F16" t="str">
-        <v/>
+      <c r="F16">
+        <v>26.25</v>
       </c>
     </row>
     <row r="17">
@@ -2772,8 +2772,8 @@
       <c r="E17">
         <v>44</v>
       </c>
-      <c r="F17" t="str">
-        <v/>
+      <c r="F17">
+        <v>27.500000000000004</v>
       </c>
     </row>
     <row r="18">
@@ -2792,8 +2792,8 @@
       <c r="E18">
         <v>42</v>
       </c>
-      <c r="F18" t="str">
-        <v/>
+      <c r="F18">
+        <v>26.25</v>
       </c>
     </row>
     <row r="19">
@@ -2812,8 +2812,8 @@
       <c r="E19">
         <v>44</v>
       </c>
-      <c r="F19" t="str">
-        <v/>
+      <c r="F19">
+        <v>27.500000000000004</v>
       </c>
     </row>
     <row r="20">
@@ -2832,8 +2832,8 @@
       <c r="E20">
         <v>46</v>
       </c>
-      <c r="F20" t="str">
-        <v/>
+      <c r="F20">
+        <v>28.749999999999996</v>
       </c>
     </row>
     <row r="21">
@@ -2852,8 +2852,8 @@
       <c r="E21">
         <v>48</v>
       </c>
-      <c r="F21" t="str">
-        <v/>
+      <c r="F21">
+        <v>30</v>
       </c>
     </row>
     <row r="22">
@@ -2872,8 +2872,8 @@
       <c r="E22">
         <v>46</v>
       </c>
-      <c r="F22" t="str">
-        <v/>
+      <c r="F22">
+        <v>28.749999999999996</v>
       </c>
     </row>
     <row r="23">
@@ -2892,8 +2892,8 @@
       <c r="E23">
         <v>48</v>
       </c>
-      <c r="F23" t="str">
-        <v/>
+      <c r="F23">
+        <v>30</v>
       </c>
     </row>
     <row r="24">
@@ -2912,8 +2912,8 @@
       <c r="E24">
         <v>50</v>
       </c>
-      <c r="F24" t="str">
-        <v/>
+      <c r="F24">
+        <v>31.25</v>
       </c>
     </row>
     <row r="25">
@@ -2932,8 +2932,8 @@
       <c r="E25">
         <v>52</v>
       </c>
-      <c r="F25" t="str">
-        <v/>
+      <c r="F25">
+        <v>32.5</v>
       </c>
     </row>
     <row r="26">
@@ -2952,8 +2952,8 @@
       <c r="E26">
         <v>38</v>
       </c>
-      <c r="F26" t="str">
-        <v/>
+      <c r="F26">
+        <v>23.75</v>
       </c>
     </row>
     <row r="27">
@@ -2972,8 +2972,8 @@
       <c r="E27">
         <v>40</v>
       </c>
-      <c r="F27" t="str">
-        <v/>
+      <c r="F27">
+        <v>25</v>
       </c>
     </row>
     <row r="28">
@@ -2992,8 +2992,8 @@
       <c r="E28">
         <v>42</v>
       </c>
-      <c r="F28" t="str">
-        <v/>
+      <c r="F28">
+        <v>26.25</v>
       </c>
     </row>
     <row r="29">
@@ -3012,8 +3012,8 @@
       <c r="E29">
         <v>44</v>
       </c>
-      <c r="F29" t="str">
-        <v/>
+      <c r="F29">
+        <v>27.500000000000004</v>
       </c>
     </row>
     <row r="30">
@@ -3032,8 +3032,8 @@
       <c r="E30">
         <v>42</v>
       </c>
-      <c r="F30" t="str">
-        <v/>
+      <c r="F30">
+        <v>26.25</v>
       </c>
     </row>
     <row r="31">
@@ -3052,8 +3052,8 @@
       <c r="E31">
         <v>44</v>
       </c>
-      <c r="F31" t="str">
-        <v/>
+      <c r="F31">
+        <v>27.500000000000004</v>
       </c>
     </row>
     <row r="32">
@@ -3072,8 +3072,8 @@
       <c r="E32">
         <v>46</v>
       </c>
-      <c r="F32" t="str">
-        <v/>
+      <c r="F32">
+        <v>28.749999999999996</v>
       </c>
     </row>
     <row r="33">
@@ -3092,8 +3092,8 @@
       <c r="E33">
         <v>48</v>
       </c>
-      <c r="F33" t="str">
-        <v/>
+      <c r="F33">
+        <v>30</v>
       </c>
     </row>
     <row r="34">
@@ -3112,8 +3112,8 @@
       <c r="E34">
         <v>46</v>
       </c>
-      <c r="F34" t="str">
-        <v/>
+      <c r="F34">
+        <v>28.749999999999996</v>
       </c>
     </row>
     <row r="35">
@@ -3132,8 +3132,8 @@
       <c r="E35">
         <v>48</v>
       </c>
-      <c r="F35" t="str">
-        <v/>
+      <c r="F35">
+        <v>30</v>
       </c>
     </row>
     <row r="36">
@@ -3152,8 +3152,8 @@
       <c r="E36">
         <v>50</v>
       </c>
-      <c r="F36" t="str">
-        <v/>
+      <c r="F36">
+        <v>31.25</v>
       </c>
     </row>
     <row r="37">
@@ -3172,8 +3172,8 @@
       <c r="E37">
         <v>52</v>
       </c>
-      <c r="F37" t="str">
-        <v/>
+      <c r="F37">
+        <v>32.5</v>
       </c>
     </row>
     <row r="38">
@@ -3192,8 +3192,8 @@
       <c r="E38">
         <v>70</v>
       </c>
-      <c r="F38" t="str">
-        <v/>
+      <c r="F38">
+        <v>43.75</v>
       </c>
     </row>
     <row r="39">
@@ -3212,8 +3212,8 @@
       <c r="E39">
         <v>72</v>
       </c>
-      <c r="F39" t="str">
-        <v/>
+      <c r="F39">
+        <v>45</v>
       </c>
     </row>
     <row r="40">
@@ -3232,8 +3232,8 @@
       <c r="E40">
         <v>74</v>
       </c>
-      <c r="F40" t="str">
-        <v/>
+      <c r="F40">
+        <v>46.25</v>
       </c>
     </row>
     <row r="41">
@@ -3252,8 +3252,8 @@
       <c r="E41">
         <v>76</v>
       </c>
-      <c r="F41" t="str">
-        <v/>
+      <c r="F41">
+        <v>47.5</v>
       </c>
     </row>
     <row r="42">
@@ -3272,8 +3272,8 @@
       <c r="E42">
         <v>78</v>
       </c>
-      <c r="F42" t="str">
-        <v/>
+      <c r="F42">
+        <v>48.75</v>
       </c>
     </row>
     <row r="43">
@@ -3292,8 +3292,8 @@
       <c r="E43">
         <v>80</v>
       </c>
-      <c r="F43" t="str">
-        <v/>
+      <c r="F43">
+        <v>50</v>
       </c>
     </row>
     <row r="44">
@@ -3312,8 +3312,8 @@
       <c r="E44">
         <v>74</v>
       </c>
-      <c r="F44" t="str">
-        <v/>
+      <c r="F44">
+        <v>46.25</v>
       </c>
     </row>
     <row r="45">
@@ -3332,8 +3332,8 @@
       <c r="E45">
         <v>76</v>
       </c>
-      <c r="F45" t="str">
-        <v/>
+      <c r="F45">
+        <v>47.5</v>
       </c>
     </row>
     <row r="46">
@@ -3352,8 +3352,8 @@
       <c r="E46">
         <v>78</v>
       </c>
-      <c r="F46" t="str">
-        <v/>
+      <c r="F46">
+        <v>48.75</v>
       </c>
     </row>
     <row r="47">
@@ -3372,8 +3372,8 @@
       <c r="E47">
         <v>80</v>
       </c>
-      <c r="F47" t="str">
-        <v/>
+      <c r="F47">
+        <v>50</v>
       </c>
     </row>
     <row r="48">
@@ -3392,8 +3392,8 @@
       <c r="E48">
         <v>82</v>
       </c>
-      <c r="F48" t="str">
-        <v/>
+      <c r="F48">
+        <v>51.24999999999999</v>
       </c>
     </row>
     <row r="49">
@@ -3412,8 +3412,8 @@
       <c r="E49">
         <v>84</v>
       </c>
-      <c r="F49" t="str">
-        <v/>
+      <c r="F49">
+        <v>52.5</v>
       </c>
     </row>
     <row r="50">
@@ -3432,8 +3432,8 @@
       <c r="E50">
         <v>78</v>
       </c>
-      <c r="F50" t="str">
-        <v/>
+      <c r="F50">
+        <v>48.75</v>
       </c>
     </row>
     <row r="51">
@@ -3452,8 +3452,8 @@
       <c r="E51">
         <v>80</v>
       </c>
-      <c r="F51" t="str">
-        <v/>
+      <c r="F51">
+        <v>50</v>
       </c>
     </row>
     <row r="52">
@@ -3472,8 +3472,8 @@
       <c r="E52">
         <v>82</v>
       </c>
-      <c r="F52" t="str">
-        <v/>
+      <c r="F52">
+        <v>51.24999999999999</v>
       </c>
     </row>
     <row r="53">
@@ -3492,8 +3492,8 @@
       <c r="E53">
         <v>84</v>
       </c>
-      <c r="F53" t="str">
-        <v/>
+      <c r="F53">
+        <v>52.5</v>
       </c>
     </row>
     <row r="54">
@@ -3512,8 +3512,8 @@
       <c r="E54">
         <v>86</v>
       </c>
-      <c r="F54" t="str">
-        <v/>
+      <c r="F54">
+        <v>53.75</v>
       </c>
     </row>
     <row r="55">
@@ -3532,8 +3532,8 @@
       <c r="E55">
         <v>88</v>
       </c>
-      <c r="F55" t="str">
-        <v/>
+      <c r="F55">
+        <v>55.00000000000001</v>
       </c>
     </row>
     <row r="56">
@@ -3552,8 +3552,8 @@
       <c r="E56">
         <v>38</v>
       </c>
-      <c r="F56" t="str">
-        <v/>
+      <c r="F56">
+        <v>23.75</v>
       </c>
     </row>
     <row r="57">
@@ -3572,8 +3572,8 @@
       <c r="E57">
         <v>40</v>
       </c>
-      <c r="F57" t="str">
-        <v/>
+      <c r="F57">
+        <v>25</v>
       </c>
     </row>
     <row r="58">
@@ -3592,8 +3592,8 @@
       <c r="E58">
         <v>42</v>
       </c>
-      <c r="F58" t="str">
-        <v/>
+      <c r="F58">
+        <v>26.25</v>
       </c>
     </row>
     <row r="59">
@@ -3612,8 +3612,8 @@
       <c r="E59">
         <v>44</v>
       </c>
-      <c r="F59" t="str">
-        <v/>
+      <c r="F59">
+        <v>27.500000000000004</v>
       </c>
     </row>
     <row r="60">
@@ -3632,8 +3632,8 @@
       <c r="E60">
         <v>42</v>
       </c>
-      <c r="F60" t="str">
-        <v/>
+      <c r="F60">
+        <v>26.25</v>
       </c>
     </row>
     <row r="61">
@@ -3652,8 +3652,8 @@
       <c r="E61">
         <v>44</v>
       </c>
-      <c r="F61" t="str">
-        <v/>
+      <c r="F61">
+        <v>27.500000000000004</v>
       </c>
     </row>
     <row r="62">
@@ -3672,8 +3672,8 @@
       <c r="E62">
         <v>46</v>
       </c>
-      <c r="F62" t="str">
-        <v/>
+      <c r="F62">
+        <v>28.749999999999996</v>
       </c>
     </row>
     <row r="63">
@@ -3692,8 +3692,8 @@
       <c r="E63">
         <v>48</v>
       </c>
-      <c r="F63" t="str">
-        <v/>
+      <c r="F63">
+        <v>30</v>
       </c>
     </row>
     <row r="64">
@@ -3712,8 +3712,8 @@
       <c r="E64">
         <v>46</v>
       </c>
-      <c r="F64" t="str">
-        <v/>
+      <c r="F64">
+        <v>28.749999999999996</v>
       </c>
     </row>
     <row r="65">
@@ -3732,8 +3732,8 @@
       <c r="E65">
         <v>48</v>
       </c>
-      <c r="F65" t="str">
-        <v/>
+      <c r="F65">
+        <v>30</v>
       </c>
     </row>
     <row r="66">
@@ -3752,8 +3752,8 @@
       <c r="E66">
         <v>50</v>
       </c>
-      <c r="F66" t="str">
-        <v/>
+      <c r="F66">
+        <v>31.25</v>
       </c>
     </row>
     <row r="67">
@@ -3772,8 +3772,8 @@
       <c r="E67">
         <v>52</v>
       </c>
-      <c r="F67" t="str">
-        <v/>
+      <c r="F67">
+        <v>32.5</v>
       </c>
     </row>
   </sheetData>
@@ -6889,7 +6889,7 @@
         <v>Não</v>
       </c>
       <c r="D61" t="str">
-        <v>Percentual informativo de 0 a 100.</v>
+        <v>Calculado automaticamente a partir de Horas, pessoa e período.</v>
       </c>
     </row>
     <row r="62">

</xml_diff>

<commit_message>
Calculate allocation capacity using eight-hour weekdays
</commit_message>
<xml_diff>
--- a/Modelo-SGP.xlsx
+++ b/Modelo-SGP.xlsx
@@ -2473,7 +2473,7 @@
         <v>38</v>
       </c>
       <c r="F2">
-        <v>23.75</v>
+        <v>21.59090909090909</v>
       </c>
     </row>
     <row r="3">
@@ -2493,7 +2493,7 @@
         <v>40</v>
       </c>
       <c r="F3">
-        <v>25</v>
+        <v>22.727272727272727</v>
       </c>
     </row>
     <row r="4">
@@ -2513,7 +2513,7 @@
         <v>42</v>
       </c>
       <c r="F4">
-        <v>26.25</v>
+        <v>23.863636363636363</v>
       </c>
     </row>
     <row r="5">
@@ -2533,7 +2533,7 @@
         <v>44</v>
       </c>
       <c r="F5">
-        <v>27.500000000000004</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
@@ -2553,7 +2553,7 @@
         <v>42</v>
       </c>
       <c r="F6">
-        <v>26.25</v>
+        <v>23.863636363636363</v>
       </c>
     </row>
     <row r="7">
@@ -2573,7 +2573,7 @@
         <v>44</v>
       </c>
       <c r="F7">
-        <v>27.500000000000004</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
@@ -2593,7 +2593,7 @@
         <v>46</v>
       </c>
       <c r="F8">
-        <v>28.749999999999996</v>
+        <v>26.136363636363637</v>
       </c>
     </row>
     <row r="9">
@@ -2613,7 +2613,7 @@
         <v>48</v>
       </c>
       <c r="F9">
-        <v>30</v>
+        <v>27.27272727272727</v>
       </c>
     </row>
     <row r="10">
@@ -2633,7 +2633,7 @@
         <v>46</v>
       </c>
       <c r="F10">
-        <v>28.749999999999996</v>
+        <v>26.136363636363637</v>
       </c>
     </row>
     <row r="11">
@@ -2653,7 +2653,7 @@
         <v>48</v>
       </c>
       <c r="F11">
-        <v>30</v>
+        <v>27.27272727272727</v>
       </c>
     </row>
     <row r="12">
@@ -2673,7 +2673,7 @@
         <v>50</v>
       </c>
       <c r="F12">
-        <v>31.25</v>
+        <v>28.40909090909091</v>
       </c>
     </row>
     <row r="13">
@@ -2693,7 +2693,7 @@
         <v>52</v>
       </c>
       <c r="F13">
-        <v>32.5</v>
+        <v>29.545454545454547</v>
       </c>
     </row>
     <row r="14">
@@ -2713,7 +2713,7 @@
         <v>38</v>
       </c>
       <c r="F14">
-        <v>23.75</v>
+        <v>21.59090909090909</v>
       </c>
     </row>
     <row r="15">
@@ -2733,7 +2733,7 @@
         <v>40</v>
       </c>
       <c r="F15">
-        <v>25</v>
+        <v>22.727272727272727</v>
       </c>
     </row>
     <row r="16">
@@ -2753,7 +2753,7 @@
         <v>42</v>
       </c>
       <c r="F16">
-        <v>26.25</v>
+        <v>23.863636363636363</v>
       </c>
     </row>
     <row r="17">
@@ -2773,7 +2773,7 @@
         <v>44</v>
       </c>
       <c r="F17">
-        <v>27.500000000000004</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18">
@@ -2793,7 +2793,7 @@
         <v>42</v>
       </c>
       <c r="F18">
-        <v>26.25</v>
+        <v>23.863636363636363</v>
       </c>
     </row>
     <row r="19">
@@ -2813,7 +2813,7 @@
         <v>44</v>
       </c>
       <c r="F19">
-        <v>27.500000000000004</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20">
@@ -2833,7 +2833,7 @@
         <v>46</v>
       </c>
       <c r="F20">
-        <v>28.749999999999996</v>
+        <v>26.136363636363637</v>
       </c>
     </row>
     <row r="21">
@@ -2853,7 +2853,7 @@
         <v>48</v>
       </c>
       <c r="F21">
-        <v>30</v>
+        <v>27.27272727272727</v>
       </c>
     </row>
     <row r="22">
@@ -2873,7 +2873,7 @@
         <v>46</v>
       </c>
       <c r="F22">
-        <v>28.749999999999996</v>
+        <v>26.136363636363637</v>
       </c>
     </row>
     <row r="23">
@@ -2893,7 +2893,7 @@
         <v>48</v>
       </c>
       <c r="F23">
-        <v>30</v>
+        <v>27.27272727272727</v>
       </c>
     </row>
     <row r="24">
@@ -2913,7 +2913,7 @@
         <v>50</v>
       </c>
       <c r="F24">
-        <v>31.25</v>
+        <v>28.40909090909091</v>
       </c>
     </row>
     <row r="25">
@@ -2933,7 +2933,7 @@
         <v>52</v>
       </c>
       <c r="F25">
-        <v>32.5</v>
+        <v>29.545454545454547</v>
       </c>
     </row>
     <row r="26">
@@ -2953,7 +2953,7 @@
         <v>38</v>
       </c>
       <c r="F26">
-        <v>23.75</v>
+        <v>21.59090909090909</v>
       </c>
     </row>
     <row r="27">
@@ -2973,7 +2973,7 @@
         <v>40</v>
       </c>
       <c r="F27">
-        <v>25</v>
+        <v>22.727272727272727</v>
       </c>
     </row>
     <row r="28">
@@ -2993,7 +2993,7 @@
         <v>42</v>
       </c>
       <c r="F28">
-        <v>26.25</v>
+        <v>23.863636363636363</v>
       </c>
     </row>
     <row r="29">
@@ -3013,7 +3013,7 @@
         <v>44</v>
       </c>
       <c r="F29">
-        <v>27.500000000000004</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30">
@@ -3033,7 +3033,7 @@
         <v>42</v>
       </c>
       <c r="F30">
-        <v>26.25</v>
+        <v>23.863636363636363</v>
       </c>
     </row>
     <row r="31">
@@ -3053,7 +3053,7 @@
         <v>44</v>
       </c>
       <c r="F31">
-        <v>27.500000000000004</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32">
@@ -3073,7 +3073,7 @@
         <v>46</v>
       </c>
       <c r="F32">
-        <v>28.749999999999996</v>
+        <v>26.136363636363637</v>
       </c>
     </row>
     <row r="33">
@@ -3093,7 +3093,7 @@
         <v>48</v>
       </c>
       <c r="F33">
-        <v>30</v>
+        <v>27.27272727272727</v>
       </c>
     </row>
     <row r="34">
@@ -3113,7 +3113,7 @@
         <v>46</v>
       </c>
       <c r="F34">
-        <v>28.749999999999996</v>
+        <v>26.136363636363637</v>
       </c>
     </row>
     <row r="35">
@@ -3133,7 +3133,7 @@
         <v>48</v>
       </c>
       <c r="F35">
-        <v>30</v>
+        <v>27.27272727272727</v>
       </c>
     </row>
     <row r="36">
@@ -3153,7 +3153,7 @@
         <v>50</v>
       </c>
       <c r="F36">
-        <v>31.25</v>
+        <v>28.40909090909091</v>
       </c>
     </row>
     <row r="37">
@@ -3173,7 +3173,7 @@
         <v>52</v>
       </c>
       <c r="F37">
-        <v>32.5</v>
+        <v>29.545454545454547</v>
       </c>
     </row>
     <row r="38">
@@ -3193,7 +3193,7 @@
         <v>70</v>
       </c>
       <c r="F38">
-        <v>43.75</v>
+        <v>39.77272727272727</v>
       </c>
     </row>
     <row r="39">
@@ -3213,7 +3213,7 @@
         <v>72</v>
       </c>
       <c r="F39">
-        <v>45</v>
+        <v>40.909090909090914</v>
       </c>
     </row>
     <row r="40">
@@ -3233,7 +3233,7 @@
         <v>74</v>
       </c>
       <c r="F40">
-        <v>46.25</v>
+        <v>42.04545454545455</v>
       </c>
     </row>
     <row r="41">
@@ -3253,7 +3253,7 @@
         <v>76</v>
       </c>
       <c r="F41">
-        <v>47.5</v>
+        <v>43.18181818181818</v>
       </c>
     </row>
     <row r="42">
@@ -3273,7 +3273,7 @@
         <v>78</v>
       </c>
       <c r="F42">
-        <v>48.75</v>
+        <v>44.31818181818182</v>
       </c>
     </row>
     <row r="43">
@@ -3293,7 +3293,7 @@
         <v>80</v>
       </c>
       <c r="F43">
-        <v>50</v>
+        <v>45.45454545454545</v>
       </c>
     </row>
     <row r="44">
@@ -3313,7 +3313,7 @@
         <v>74</v>
       </c>
       <c r="F44">
-        <v>46.25</v>
+        <v>42.04545454545455</v>
       </c>
     </row>
     <row r="45">
@@ -3333,7 +3333,7 @@
         <v>76</v>
       </c>
       <c r="F45">
-        <v>47.5</v>
+        <v>43.18181818181818</v>
       </c>
     </row>
     <row r="46">
@@ -3353,7 +3353,7 @@
         <v>78</v>
       </c>
       <c r="F46">
-        <v>48.75</v>
+        <v>44.31818181818182</v>
       </c>
     </row>
     <row r="47">
@@ -3373,7 +3373,7 @@
         <v>80</v>
       </c>
       <c r="F47">
-        <v>50</v>
+        <v>45.45454545454545</v>
       </c>
     </row>
     <row r="48">
@@ -3393,7 +3393,7 @@
         <v>82</v>
       </c>
       <c r="F48">
-        <v>51.24999999999999</v>
+        <v>46.590909090909086</v>
       </c>
     </row>
     <row r="49">
@@ -3413,7 +3413,7 @@
         <v>84</v>
       </c>
       <c r="F49">
-        <v>52.5</v>
+        <v>47.72727272727273</v>
       </c>
     </row>
     <row r="50">
@@ -3433,7 +3433,7 @@
         <v>78</v>
       </c>
       <c r="F50">
-        <v>48.75</v>
+        <v>44.31818181818182</v>
       </c>
     </row>
     <row r="51">
@@ -3453,7 +3453,7 @@
         <v>80</v>
       </c>
       <c r="F51">
-        <v>50</v>
+        <v>45.45454545454545</v>
       </c>
     </row>
     <row r="52">
@@ -3473,7 +3473,7 @@
         <v>82</v>
       </c>
       <c r="F52">
-        <v>51.24999999999999</v>
+        <v>46.590909090909086</v>
       </c>
     </row>
     <row r="53">
@@ -3493,7 +3493,7 @@
         <v>84</v>
       </c>
       <c r="F53">
-        <v>52.5</v>
+        <v>47.72727272727273</v>
       </c>
     </row>
     <row r="54">
@@ -3513,7 +3513,7 @@
         <v>86</v>
       </c>
       <c r="F54">
-        <v>53.75</v>
+        <v>48.86363636363637</v>
       </c>
     </row>
     <row r="55">
@@ -3533,7 +3533,7 @@
         <v>88</v>
       </c>
       <c r="F55">
-        <v>55.00000000000001</v>
+        <v>50</v>
       </c>
     </row>
     <row r="56">
@@ -3553,7 +3553,7 @@
         <v>38</v>
       </c>
       <c r="F56">
-        <v>23.75</v>
+        <v>21.59090909090909</v>
       </c>
     </row>
     <row r="57">
@@ -3573,7 +3573,7 @@
         <v>40</v>
       </c>
       <c r="F57">
-        <v>25</v>
+        <v>22.727272727272727</v>
       </c>
     </row>
     <row r="58">
@@ -3593,7 +3593,7 @@
         <v>42</v>
       </c>
       <c r="F58">
-        <v>26.25</v>
+        <v>23.863636363636363</v>
       </c>
     </row>
     <row r="59">
@@ -3613,7 +3613,7 @@
         <v>44</v>
       </c>
       <c r="F59">
-        <v>27.500000000000004</v>
+        <v>25</v>
       </c>
     </row>
     <row r="60">
@@ -3633,7 +3633,7 @@
         <v>42</v>
       </c>
       <c r="F60">
-        <v>26.25</v>
+        <v>23.863636363636363</v>
       </c>
     </row>
     <row r="61">
@@ -3653,7 +3653,7 @@
         <v>44</v>
       </c>
       <c r="F61">
-        <v>27.500000000000004</v>
+        <v>25</v>
       </c>
     </row>
     <row r="62">
@@ -3673,7 +3673,7 @@
         <v>46</v>
       </c>
       <c r="F62">
-        <v>28.749999999999996</v>
+        <v>26.136363636363637</v>
       </c>
     </row>
     <row r="63">
@@ -3693,7 +3693,7 @@
         <v>48</v>
       </c>
       <c r="F63">
-        <v>30</v>
+        <v>27.27272727272727</v>
       </c>
     </row>
     <row r="64">
@@ -3713,7 +3713,7 @@
         <v>46</v>
       </c>
       <c r="F64">
-        <v>28.749999999999996</v>
+        <v>26.136363636363637</v>
       </c>
     </row>
     <row r="65">
@@ -3733,7 +3733,7 @@
         <v>48</v>
       </c>
       <c r="F65">
-        <v>30</v>
+        <v>27.27272727272727</v>
       </c>
     </row>
     <row r="66">
@@ -3753,7 +3753,7 @@
         <v>50</v>
       </c>
       <c r="F66">
-        <v>31.25</v>
+        <v>28.40909090909091</v>
       </c>
     </row>
     <row r="67">
@@ -3773,7 +3773,7 @@
         <v>52</v>
       </c>
       <c r="F67">
-        <v>32.5</v>
+        <v>29.545454545454547</v>
       </c>
     </row>
   </sheetData>
@@ -6267,7 +6267,7 @@
         <v>Capacidade</v>
       </c>
       <c r="B14" t="str">
-        <v>Capacidade mensal em horas, proporcional aos dias corridos do mês. Horas alocadas são totais do intervalo, distribuídas uniformemente pelos dias corridos. Feriados não são descontados. Percentual é informativo; Horas alimenta a capacidade.</v>
+        <v>Capacidade = dias de segunda a sexta no período × 8h. Horas distribuídas apenas nesses dias. Percentual = horas / capacidade do intervalo × 100. Feriados e férias não são descontados. A coluna Capacidade Mensal é legada e não participa dos cálculos.</v>
       </c>
     </row>
     <row r="15">
@@ -6785,7 +6785,7 @@
         <v>Sim</v>
       </c>
       <c r="D53" t="str">
-        <v>Capacidade mensal em horas; número não negativo.</v>
+        <v>Campo legado mantido por compatibilidade. Não altera os cálculos: a jornada é de 8h por dia, de segunda a sexta.</v>
       </c>
     </row>
     <row r="54">

</xml_diff>

<commit_message>
Plan demand schedules and effort through project phases
</commit_message>
<xml_diff>
--- a/Modelo-SGP.xlsx
+++ b/Modelo-SGP.xlsx
@@ -11,10 +11,10 @@
     <sheet name="LEIA-ME" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Demandas!$A$1:$AC$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Demandas!$A$1:$AE$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">Pessoas!$A$1:$G$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2">Alocacoes!$A$1:$F$67</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3">Fases!$A$1:$E$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3">Fases!$A$1:$G$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4">Marcos!$A$1:$E$46</definedName>
   </definedNames>
 </workbook>
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC16"/>
+  <dimension ref="A1:AE16"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
@@ -429,17 +429,19 @@
     <col min="16" max="16" width="18.83203125" customWidth="1"/>
     <col min="17" max="17" width="18.83203125" customWidth="1"/>
     <col min="18" max="18" width="21.83203125" customWidth="1"/>
-    <col min="19" max="19" width="17.83203125" customWidth="1"/>
-    <col min="20" max="20" width="18.83203125" customWidth="1"/>
-    <col min="21" max="21" width="25.83203125" customWidth="1"/>
-    <col min="22" max="22" width="17.83203125" customWidth="1"/>
-    <col min="23" max="23" width="20.83203125" customWidth="1"/>
+    <col min="19" max="19" width="24.83203125" customWidth="1"/>
+    <col min="20" max="20" width="30.83203125" customWidth="1"/>
+    <col min="21" max="21" width="17.83203125" customWidth="1"/>
+    <col min="22" max="22" width="18.83203125" customWidth="1"/>
+    <col min="23" max="23" width="25.83203125" customWidth="1"/>
     <col min="24" max="24" width="17.83203125" customWidth="1"/>
-    <col min="25" max="25" width="30.83203125" customWidth="1"/>
+    <col min="25" max="25" width="20.83203125" customWidth="1"/>
     <col min="26" max="26" width="17.83203125" customWidth="1"/>
-    <col min="27" max="27" width="20.83203125" customWidth="1"/>
+    <col min="27" max="27" width="30.83203125" customWidth="1"/>
     <col min="28" max="28" width="17.83203125" customWidth="1"/>
-    <col min="29" max="29" width="17.83203125" customWidth="1"/>
+    <col min="29" max="29" width="20.83203125" customWidth="1"/>
+    <col min="30" max="30" width="17.83203125" customWidth="1"/>
+    <col min="31" max="31" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,36 +500,42 @@
         <v>Data Final Prevista</v>
       </c>
       <c r="S1" t="str">
+        <v>Cronograma pelas fases</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Entrega acordada com cliente</v>
+      </c>
+      <c r="U1" t="str">
         <v>Horas Estimadas</v>
       </c>
-      <c r="T1" t="str">
+      <c r="V1" t="str">
         <v>Horas Consumidas</v>
       </c>
-      <c r="U1" t="str">
+      <c r="W1" t="str">
         <v>Percentual de Conclusão</v>
       </c>
-      <c r="V1" t="str">
+      <c r="X1" t="str">
         <v>Próximo Marco</v>
       </c>
-      <c r="W1" t="str">
+      <c r="Y1" t="str">
         <v>Data Próximo Marco</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Z1" t="str">
         <v>Dependência</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="AA1" t="str">
         <v>Responsável pela Dependência</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AB1" t="str">
         <v>Risco</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AC1" t="str">
         <v>Descrição do Risco</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AD1" t="str">
         <v>Link Git</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AE1" t="str">
         <v>Observação</v>
       </c>
     </row>
@@ -586,37 +594,43 @@
       <c r="R2" t="str">
         <v>2026-10-09</v>
       </c>
-      <c r="S2">
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2">
         <v>240</v>
       </c>
-      <c r="T2">
+      <c r="V2">
         <v>120</v>
       </c>
-      <c r="U2">
+      <c r="W2">
         <v>45</v>
       </c>
-      <c r="V2" t="str">
+      <c r="X2" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W2" t="str">
+      <c r="Y2" t="str">
         <v>2026-09-24</v>
       </c>
-      <c r="X2" t="str">
-        <v/>
-      </c>
-      <c r="Y2" t="str">
-        <v/>
-      </c>
       <c r="Z2" t="str">
+        <v/>
+      </c>
+      <c r="AA2" t="str">
+        <v/>
+      </c>
+      <c r="AB2" t="str">
         <v>Nenhum</v>
       </c>
-      <c r="AA2" t="str">
-        <v/>
-      </c>
-      <c r="AB2" t="str">
-        <v/>
-      </c>
       <c r="AC2" t="str">
+        <v/>
+      </c>
+      <c r="AD2" t="str">
+        <v/>
+      </c>
+      <c r="AE2" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
@@ -675,37 +689,43 @@
       <c r="R3" t="str">
         <v>2026-11-13</v>
       </c>
-      <c r="S3">
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3">
         <v>320</v>
       </c>
-      <c r="T3">
+      <c r="V3">
         <v>120</v>
       </c>
-      <c r="U3">
+      <c r="W3">
         <v>45</v>
       </c>
-      <c r="V3" t="str">
+      <c r="X3" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W3" t="str">
+      <c r="Y3" t="str">
         <v>2026-10-29</v>
       </c>
-      <c r="X3" t="str">
-        <v/>
-      </c>
-      <c r="Y3" t="str">
-        <v/>
-      </c>
       <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v/>
+      </c>
+      <c r="AB3" t="str">
         <v>Nenhum</v>
       </c>
-      <c r="AA3" t="str">
-        <v/>
-      </c>
-      <c r="AB3" t="str">
-        <v/>
-      </c>
       <c r="AC3" t="str">
+        <v/>
+      </c>
+      <c r="AD3" t="str">
+        <v/>
+      </c>
+      <c r="AE3" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
@@ -764,37 +784,43 @@
       <c r="R4" t="str">
         <v>2026-12-18</v>
       </c>
-      <c r="S4">
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4">
         <v>400</v>
       </c>
-      <c r="T4">
+      <c r="V4">
         <v>0</v>
       </c>
-      <c r="U4">
+      <c r="W4">
         <v>0</v>
       </c>
-      <c r="V4" t="str">
+      <c r="X4" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W4" t="str">
+      <c r="Y4" t="str">
         <v>2026-12-03</v>
       </c>
-      <c r="X4" t="str">
-        <v/>
-      </c>
-      <c r="Y4" t="str">
-        <v/>
-      </c>
       <c r="Z4" t="str">
+        <v/>
+      </c>
+      <c r="AA4" t="str">
+        <v/>
+      </c>
+      <c r="AB4" t="str">
         <v>Nenhum</v>
       </c>
-      <c r="AA4" t="str">
-        <v/>
-      </c>
-      <c r="AB4" t="str">
-        <v/>
-      </c>
       <c r="AC4" t="str">
+        <v/>
+      </c>
+      <c r="AD4" t="str">
+        <v/>
+      </c>
+      <c r="AE4" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
@@ -853,37 +879,43 @@
       <c r="R5" t="str">
         <v>2026-10-12</v>
       </c>
-      <c r="S5">
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5">
         <v>240</v>
       </c>
-      <c r="T5">
+      <c r="V5">
         <v>120</v>
       </c>
-      <c r="U5">
+      <c r="W5">
         <v>45</v>
       </c>
-      <c r="V5" t="str">
+      <c r="X5" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W5" t="str">
+      <c r="Y5" t="str">
         <v>2026-09-27</v>
       </c>
-      <c r="X5" t="str">
-        <v/>
-      </c>
-      <c r="Y5" t="str">
-        <v/>
-      </c>
       <c r="Z5" t="str">
+        <v/>
+      </c>
+      <c r="AA5" t="str">
+        <v/>
+      </c>
+      <c r="AB5" t="str">
         <v>Nenhum</v>
       </c>
-      <c r="AA5" t="str">
-        <v/>
-      </c>
-      <c r="AB5" t="str">
-        <v/>
-      </c>
       <c r="AC5" t="str">
+        <v/>
+      </c>
+      <c r="AD5" t="str">
+        <v/>
+      </c>
+      <c r="AE5" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
@@ -942,37 +974,43 @@
       <c r="R6" t="str">
         <v>2026-11-16</v>
       </c>
-      <c r="S6">
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6">
         <v>320</v>
       </c>
-      <c r="T6">
+      <c r="V6">
         <v>120</v>
       </c>
-      <c r="U6">
+      <c r="W6">
         <v>45</v>
       </c>
-      <c r="V6" t="str">
+      <c r="X6" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W6" t="str">
+      <c r="Y6" t="str">
         <v>2026-11-01</v>
       </c>
-      <c r="X6" t="str">
+      <c r="Z6" t="str">
         <v>Validação do cliente</v>
       </c>
-      <c r="Y6" t="str">
+      <c r="AA6" t="str">
         <v>Plan</v>
       </c>
-      <c r="Z6" t="str">
+      <c r="AB6" t="str">
         <v>Média</v>
       </c>
-      <c r="AA6" t="str">
+      <c r="AC6" t="str">
         <v>Decisão do cliente necessária para avançar.</v>
       </c>
-      <c r="AB6" t="str">
-        <v/>
-      </c>
-      <c r="AC6" t="str">
+      <c r="AD6" t="str">
+        <v/>
+      </c>
+      <c r="AE6" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
@@ -1031,37 +1069,43 @@
       <c r="R7" t="str">
         <v>2026-12-21</v>
       </c>
-      <c r="S7">
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7">
         <v>400</v>
       </c>
-      <c r="T7">
+      <c r="V7">
         <v>0</v>
       </c>
-      <c r="U7">
+      <c r="W7">
         <v>0</v>
       </c>
-      <c r="V7" t="str">
+      <c r="X7" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W7" t="str">
+      <c r="Y7" t="str">
         <v>2026-12-06</v>
       </c>
-      <c r="X7" t="str">
-        <v/>
-      </c>
-      <c r="Y7" t="str">
-        <v/>
-      </c>
       <c r="Z7" t="str">
+        <v/>
+      </c>
+      <c r="AA7" t="str">
+        <v/>
+      </c>
+      <c r="AB7" t="str">
         <v>Nenhum</v>
       </c>
-      <c r="AA7" t="str">
-        <v/>
-      </c>
-      <c r="AB7" t="str">
-        <v/>
-      </c>
       <c r="AC7" t="str">
+        <v/>
+      </c>
+      <c r="AD7" t="str">
+        <v/>
+      </c>
+      <c r="AE7" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
@@ -1120,37 +1164,43 @@
       <c r="R8" t="str">
         <v>2026-10-15</v>
       </c>
-      <c r="S8">
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8">
         <v>240</v>
       </c>
-      <c r="T8">
+      <c r="V8">
         <v>120</v>
       </c>
-      <c r="U8">
+      <c r="W8">
         <v>45</v>
       </c>
-      <c r="V8" t="str">
+      <c r="X8" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W8" t="str">
+      <c r="Y8" t="str">
         <v>2026-09-30</v>
       </c>
-      <c r="X8" t="str">
-        <v/>
-      </c>
-      <c r="Y8" t="str">
-        <v/>
-      </c>
       <c r="Z8" t="str">
+        <v/>
+      </c>
+      <c r="AA8" t="str">
+        <v/>
+      </c>
+      <c r="AB8" t="str">
         <v>Nenhum</v>
       </c>
-      <c r="AA8" t="str">
-        <v/>
-      </c>
-      <c r="AB8" t="str">
-        <v/>
-      </c>
       <c r="AC8" t="str">
+        <v/>
+      </c>
+      <c r="AD8" t="str">
+        <v/>
+      </c>
+      <c r="AE8" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
@@ -1209,37 +1259,43 @@
       <c r="R9" t="str">
         <v>2026-11-19</v>
       </c>
-      <c r="S9">
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9">
         <v>320</v>
       </c>
-      <c r="T9">
+      <c r="V9">
         <v>120</v>
       </c>
-      <c r="U9">
+      <c r="W9">
         <v>45</v>
       </c>
-      <c r="V9" t="str">
+      <c r="X9" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W9" t="str">
+      <c r="Y9" t="str">
         <v>2026-11-04</v>
       </c>
-      <c r="X9" t="str">
+      <c r="Z9" t="str">
         <v>Validação do cliente</v>
       </c>
-      <c r="Y9" t="str">
+      <c r="AA9" t="str">
         <v>Plan</v>
       </c>
-      <c r="Z9" t="str">
+      <c r="AB9" t="str">
         <v>Média</v>
       </c>
-      <c r="AA9" t="str">
+      <c r="AC9" t="str">
         <v>Decisão do cliente necessária para avançar.</v>
       </c>
-      <c r="AB9" t="str">
-        <v/>
-      </c>
-      <c r="AC9" t="str">
+      <c r="AD9" t="str">
+        <v/>
+      </c>
+      <c r="AE9" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
@@ -1298,37 +1354,43 @@
       <c r="R10" t="str">
         <v>2026-12-24</v>
       </c>
-      <c r="S10">
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10">
         <v>400</v>
       </c>
-      <c r="T10">
+      <c r="V10">
         <v>0</v>
       </c>
-      <c r="U10">
+      <c r="W10">
         <v>0</v>
       </c>
-      <c r="V10" t="str">
+      <c r="X10" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W10" t="str">
+      <c r="Y10" t="str">
         <v>2026-12-09</v>
       </c>
-      <c r="X10" t="str">
-        <v/>
-      </c>
-      <c r="Y10" t="str">
-        <v/>
-      </c>
       <c r="Z10" t="str">
+        <v/>
+      </c>
+      <c r="AA10" t="str">
+        <v/>
+      </c>
+      <c r="AB10" t="str">
         <v>Nenhum</v>
       </c>
-      <c r="AA10" t="str">
-        <v/>
-      </c>
-      <c r="AB10" t="str">
-        <v/>
-      </c>
       <c r="AC10" t="str">
+        <v/>
+      </c>
+      <c r="AD10" t="str">
+        <v/>
+      </c>
+      <c r="AE10" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
@@ -1387,37 +1449,43 @@
       <c r="R11" t="str">
         <v>2026-10-18</v>
       </c>
-      <c r="S11">
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11">
         <v>240</v>
       </c>
-      <c r="T11">
+      <c r="V11">
         <v>120</v>
       </c>
-      <c r="U11">
+      <c r="W11">
         <v>45</v>
       </c>
-      <c r="V11" t="str">
+      <c r="X11" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W11" t="str">
+      <c r="Y11" t="str">
         <v>2026-10-03</v>
       </c>
-      <c r="X11" t="str">
-        <v/>
-      </c>
-      <c r="Y11" t="str">
-        <v/>
-      </c>
       <c r="Z11" t="str">
+        <v/>
+      </c>
+      <c r="AA11" t="str">
+        <v/>
+      </c>
+      <c r="AB11" t="str">
         <v>Nenhum</v>
       </c>
-      <c r="AA11" t="str">
-        <v/>
-      </c>
-      <c r="AB11" t="str">
-        <v/>
-      </c>
       <c r="AC11" t="str">
+        <v/>
+      </c>
+      <c r="AD11" t="str">
+        <v/>
+      </c>
+      <c r="AE11" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
@@ -1476,37 +1544,43 @@
       <c r="R12" t="str">
         <v>2026-11-22</v>
       </c>
-      <c r="S12">
+      <c r="S12" t="str">
+        <v/>
+      </c>
+      <c r="T12" t="str">
+        <v/>
+      </c>
+      <c r="U12">
         <v>320</v>
       </c>
-      <c r="T12">
+      <c r="V12">
         <v>120</v>
       </c>
-      <c r="U12">
+      <c r="W12">
         <v>45</v>
       </c>
-      <c r="V12" t="str">
+      <c r="X12" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W12" t="str">
+      <c r="Y12" t="str">
         <v>2026-11-07</v>
       </c>
-      <c r="X12" t="str">
-        <v/>
-      </c>
-      <c r="Y12" t="str">
-        <v/>
-      </c>
       <c r="Z12" t="str">
+        <v/>
+      </c>
+      <c r="AA12" t="str">
+        <v/>
+      </c>
+      <c r="AB12" t="str">
         <v>Alta</v>
       </c>
-      <c r="AA12" t="str">
+      <c r="AC12" t="str">
         <v>Equipe acima da capacidade no período.</v>
       </c>
-      <c r="AB12" t="str">
-        <v/>
-      </c>
-      <c r="AC12" t="str">
+      <c r="AD12" t="str">
+        <v/>
+      </c>
+      <c r="AE12" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
@@ -1565,37 +1639,43 @@
       <c r="R13" t="str">
         <v>2026-12-27</v>
       </c>
-      <c r="S13">
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13">
         <v>400</v>
       </c>
-      <c r="T13">
+      <c r="V13">
         <v>0</v>
       </c>
-      <c r="U13">
+      <c r="W13">
         <v>0</v>
       </c>
-      <c r="V13" t="str">
+      <c r="X13" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W13" t="str">
+      <c r="Y13" t="str">
         <v>2026-12-12</v>
       </c>
-      <c r="X13" t="str">
-        <v/>
-      </c>
-      <c r="Y13" t="str">
-        <v/>
-      </c>
       <c r="Z13" t="str">
+        <v/>
+      </c>
+      <c r="AA13" t="str">
+        <v/>
+      </c>
+      <c r="AB13" t="str">
         <v>Nenhum</v>
       </c>
-      <c r="AA13" t="str">
-        <v/>
-      </c>
-      <c r="AB13" t="str">
-        <v/>
-      </c>
       <c r="AC13" t="str">
+        <v/>
+      </c>
+      <c r="AD13" t="str">
+        <v/>
+      </c>
+      <c r="AE13" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
@@ -1654,37 +1734,43 @@
       <c r="R14" t="str">
         <v>2026-10-21</v>
       </c>
-      <c r="S14">
+      <c r="S14" t="str">
+        <v/>
+      </c>
+      <c r="T14" t="str">
+        <v/>
+      </c>
+      <c r="U14">
         <v>240</v>
       </c>
-      <c r="T14">
+      <c r="V14">
         <v>120</v>
       </c>
-      <c r="U14">
+      <c r="W14">
         <v>45</v>
       </c>
-      <c r="V14" t="str">
+      <c r="X14" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W14" t="str">
+      <c r="Y14" t="str">
         <v>2026-10-06</v>
       </c>
-      <c r="X14" t="str">
-        <v/>
-      </c>
-      <c r="Y14" t="str">
-        <v/>
-      </c>
       <c r="Z14" t="str">
+        <v/>
+      </c>
+      <c r="AA14" t="str">
+        <v/>
+      </c>
+      <c r="AB14" t="str">
         <v>Nenhum</v>
       </c>
-      <c r="AA14" t="str">
-        <v/>
-      </c>
-      <c r="AB14" t="str">
-        <v/>
-      </c>
       <c r="AC14" t="str">
+        <v/>
+      </c>
+      <c r="AD14" t="str">
+        <v/>
+      </c>
+      <c r="AE14" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
@@ -1743,37 +1829,43 @@
       <c r="R15" t="str">
         <v>2026-11-25</v>
       </c>
-      <c r="S15">
+      <c r="S15" t="str">
+        <v/>
+      </c>
+      <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15">
         <v>320</v>
       </c>
-      <c r="T15">
+      <c r="V15">
         <v>120</v>
       </c>
-      <c r="U15">
+      <c r="W15">
         <v>45</v>
       </c>
-      <c r="V15" t="str">
+      <c r="X15" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W15" t="str">
+      <c r="Y15" t="str">
         <v>2026-11-10</v>
       </c>
-      <c r="X15" t="str">
-        <v/>
-      </c>
-      <c r="Y15" t="str">
-        <v/>
-      </c>
       <c r="Z15" t="str">
+        <v/>
+      </c>
+      <c r="AA15" t="str">
+        <v/>
+      </c>
+      <c r="AB15" t="str">
         <v>Nenhum</v>
       </c>
-      <c r="AA15" t="str">
-        <v/>
-      </c>
-      <c r="AB15" t="str">
-        <v/>
-      </c>
       <c r="AC15" t="str">
+        <v/>
+      </c>
+      <c r="AD15" t="str">
+        <v/>
+      </c>
+      <c r="AE15" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
@@ -1832,44 +1924,50 @@
       <c r="R16" t="str">
         <v>2026-12-30</v>
       </c>
-      <c r="S16">
+      <c r="S16" t="str">
+        <v/>
+      </c>
+      <c r="T16" t="str">
+        <v/>
+      </c>
+      <c r="U16">
         <v>400</v>
       </c>
-      <c r="T16">
+      <c r="V16">
         <v>0</v>
       </c>
-      <c r="U16">
+      <c r="W16">
         <v>0</v>
       </c>
-      <c r="V16" t="str">
+      <c r="X16" t="str">
         <v>Entrega técnica</v>
       </c>
-      <c r="W16" t="str">
+      <c r="Y16" t="str">
         <v>2026-12-15</v>
       </c>
-      <c r="X16" t="str">
-        <v/>
-      </c>
-      <c r="Y16" t="str">
-        <v/>
-      </c>
       <c r="Z16" t="str">
+        <v/>
+      </c>
+      <c r="AA16" t="str">
+        <v/>
+      </c>
+      <c r="AB16" t="str">
         <v>Nenhum</v>
       </c>
-      <c r="AA16" t="str">
-        <v/>
-      </c>
-      <c r="AB16" t="str">
-        <v/>
-      </c>
       <c r="AC16" t="str">
+        <v/>
+      </c>
+      <c r="AD16" t="str">
+        <v/>
+      </c>
+      <c r="AE16" t="str">
         <v>Dados fictícios para demonstração.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC16"/>
+  <autoFilter ref="A1:AE16"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3786,13 +3884,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E91"/>
+  <dimension ref="A1:G91"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
     <col min="3" max="3" width="17.83203125" customWidth="1"/>
     <col min="4" max="4" width="17.83203125" customWidth="1"/>
     <col min="5" max="5" width="17.83203125" customWidth="1"/>
+    <col min="6" max="6" width="29.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3811,6 +3911,12 @@
       <c r="E1" t="str">
         <v>Status</v>
       </c>
+      <c r="F1" t="str">
+        <v>Consome horas da estimativa</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Horas planejadas</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -3828,6 +3934,12 @@
       <c r="E2" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -3845,6 +3957,12 @@
       <c r="E3" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -3862,6 +3980,12 @@
       <c r="E4" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -3879,6 +4003,12 @@
       <c r="E5" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -3896,6 +4026,12 @@
       <c r="E6" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -3913,6 +4049,12 @@
       <c r="E7" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -3930,6 +4072,12 @@
       <c r="E8" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -3947,6 +4095,12 @@
       <c r="E9" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -3964,6 +4118,12 @@
       <c r="E10" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -3981,6 +4141,12 @@
       <c r="E11" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -3998,6 +4164,12 @@
       <c r="E12" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -4015,6 +4187,12 @@
       <c r="E13" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -4032,6 +4210,12 @@
       <c r="E14" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -4049,6 +4233,12 @@
       <c r="E15" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -4066,6 +4256,12 @@
       <c r="E16" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -4083,6 +4279,12 @@
       <c r="E17" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -4100,6 +4302,12 @@
       <c r="E18" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -4117,6 +4325,12 @@
       <c r="E19" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -4134,6 +4348,12 @@
       <c r="E20" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -4151,6 +4371,12 @@
       <c r="E21" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -4168,6 +4394,12 @@
       <c r="E22" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -4185,6 +4417,12 @@
       <c r="E23" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -4202,6 +4440,12 @@
       <c r="E24" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -4219,6 +4463,12 @@
       <c r="E25" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -4236,6 +4486,12 @@
       <c r="E26" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -4253,6 +4509,12 @@
       <c r="E27" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -4270,6 +4532,12 @@
       <c r="E28" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -4287,6 +4555,12 @@
       <c r="E29" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -4304,6 +4578,12 @@
       <c r="E30" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -4321,6 +4601,12 @@
       <c r="E31" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F31" t="str">
+        <v/>
+      </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -4338,6 +4624,12 @@
       <c r="E32" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F32" t="str">
+        <v/>
+      </c>
+      <c r="G32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -4355,6 +4647,12 @@
       <c r="E33" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -4372,6 +4670,12 @@
       <c r="E34" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -4389,6 +4693,12 @@
       <c r="E35" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -4406,6 +4716,12 @@
       <c r="E36" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -4423,6 +4739,12 @@
       <c r="E37" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -4440,6 +4762,12 @@
       <c r="E38" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -4457,6 +4785,12 @@
       <c r="E39" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
+      <c r="G39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -4474,6 +4808,12 @@
       <c r="E40" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -4491,6 +4831,12 @@
       <c r="E41" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -4508,6 +4854,12 @@
       <c r="E42" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -4525,6 +4877,12 @@
       <c r="E43" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -4542,6 +4900,12 @@
       <c r="E44" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -4559,6 +4923,12 @@
       <c r="E45" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F45" t="str">
+        <v/>
+      </c>
+      <c r="G45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -4576,6 +4946,12 @@
       <c r="E46" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F46" t="str">
+        <v/>
+      </c>
+      <c r="G46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -4593,6 +4969,12 @@
       <c r="E47" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -4610,6 +4992,12 @@
       <c r="E48" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+      <c r="G48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -4627,6 +5015,12 @@
       <c r="E49" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+      <c r="G49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -4644,6 +5038,12 @@
       <c r="E50" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F50" t="str">
+        <v/>
+      </c>
+      <c r="G50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -4661,6 +5061,12 @@
       <c r="E51" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+      <c r="G51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -4678,6 +5084,12 @@
       <c r="E52" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+      <c r="G52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -4695,6 +5107,12 @@
       <c r="E53" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F53" t="str">
+        <v/>
+      </c>
+      <c r="G53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -4712,6 +5130,12 @@
       <c r="E54" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F54" t="str">
+        <v/>
+      </c>
+      <c r="G54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -4729,6 +5153,12 @@
       <c r="E55" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F55" t="str">
+        <v/>
+      </c>
+      <c r="G55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -4746,6 +5176,12 @@
       <c r="E56" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F56" t="str">
+        <v/>
+      </c>
+      <c r="G56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -4763,6 +5199,12 @@
       <c r="E57" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+      <c r="G57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -4780,6 +5222,12 @@
       <c r="E58" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F58" t="str">
+        <v/>
+      </c>
+      <c r="G58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -4797,6 +5245,12 @@
       <c r="E59" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F59" t="str">
+        <v/>
+      </c>
+      <c r="G59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -4814,6 +5268,12 @@
       <c r="E60" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F60" t="str">
+        <v/>
+      </c>
+      <c r="G60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -4831,6 +5291,12 @@
       <c r="E61" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F61" t="str">
+        <v/>
+      </c>
+      <c r="G61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -4848,6 +5314,12 @@
       <c r="E62" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F62" t="str">
+        <v/>
+      </c>
+      <c r="G62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -4865,6 +5337,12 @@
       <c r="E63" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F63" t="str">
+        <v/>
+      </c>
+      <c r="G63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -4882,6 +5360,12 @@
       <c r="E64" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F64" t="str">
+        <v/>
+      </c>
+      <c r="G64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -4899,6 +5383,12 @@
       <c r="E65" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F65" t="str">
+        <v/>
+      </c>
+      <c r="G65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -4916,6 +5406,12 @@
       <c r="E66" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F66" t="str">
+        <v/>
+      </c>
+      <c r="G66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -4933,6 +5429,12 @@
       <c r="E67" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F67" t="str">
+        <v/>
+      </c>
+      <c r="G67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -4950,6 +5452,12 @@
       <c r="E68" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F68" t="str">
+        <v/>
+      </c>
+      <c r="G68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -4967,6 +5475,12 @@
       <c r="E69" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F69" t="str">
+        <v/>
+      </c>
+      <c r="G69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -4984,6 +5498,12 @@
       <c r="E70" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F70" t="str">
+        <v/>
+      </c>
+      <c r="G70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -5001,6 +5521,12 @@
       <c r="E71" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F71" t="str">
+        <v/>
+      </c>
+      <c r="G71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -5018,6 +5544,12 @@
       <c r="E72" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F72" t="str">
+        <v/>
+      </c>
+      <c r="G72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -5035,6 +5567,12 @@
       <c r="E73" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F73" t="str">
+        <v/>
+      </c>
+      <c r="G73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -5052,6 +5590,12 @@
       <c r="E74" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F74" t="str">
+        <v/>
+      </c>
+      <c r="G74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -5069,6 +5613,12 @@
       <c r="E75" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F75" t="str">
+        <v/>
+      </c>
+      <c r="G75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -5086,6 +5636,12 @@
       <c r="E76" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F76" t="str">
+        <v/>
+      </c>
+      <c r="G76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -5103,6 +5659,12 @@
       <c r="E77" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F77" t="str">
+        <v/>
+      </c>
+      <c r="G77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -5120,6 +5682,12 @@
       <c r="E78" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F78" t="str">
+        <v/>
+      </c>
+      <c r="G78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -5137,6 +5705,12 @@
       <c r="E79" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F79" t="str">
+        <v/>
+      </c>
+      <c r="G79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -5154,6 +5728,12 @@
       <c r="E80" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F80" t="str">
+        <v/>
+      </c>
+      <c r="G80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -5171,6 +5751,12 @@
       <c r="E81" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F81" t="str">
+        <v/>
+      </c>
+      <c r="G81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -5188,6 +5774,12 @@
       <c r="E82" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F82" t="str">
+        <v/>
+      </c>
+      <c r="G82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -5205,6 +5797,12 @@
       <c r="E83" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F83" t="str">
+        <v/>
+      </c>
+      <c r="G83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -5222,6 +5820,12 @@
       <c r="E84" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F84" t="str">
+        <v/>
+      </c>
+      <c r="G84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -5239,6 +5843,12 @@
       <c r="E85" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F85" t="str">
+        <v/>
+      </c>
+      <c r="G85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -5256,6 +5866,12 @@
       <c r="E86" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F86" t="str">
+        <v/>
+      </c>
+      <c r="G86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -5273,6 +5889,12 @@
       <c r="E87" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F87" t="str">
+        <v/>
+      </c>
+      <c r="G87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -5290,6 +5912,12 @@
       <c r="E88" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F88" t="str">
+        <v/>
+      </c>
+      <c r="G88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -5307,6 +5935,12 @@
       <c r="E89" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F89" t="str">
+        <v/>
+      </c>
+      <c r="G89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -5324,6 +5958,12 @@
       <c r="E90" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F90" t="str">
+        <v/>
+      </c>
+      <c r="G90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -5341,11 +5981,17 @@
       <c r="E91" t="str">
         <v>Em andamento</v>
       </c>
+      <c r="F91" t="str">
+        <v/>
+      </c>
+      <c r="G91" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E91"/>
+  <autoFilter ref="A1:G91"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E91"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G91"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6153,7 +6799,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D78"/>
+  <dimension ref="A1:D82"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -6482,7 +7128,7 @@
         <v>start</v>
       </c>
       <c r="C31" t="str">
-        <v>Sim</v>
+        <v>Não</v>
       </c>
       <c r="D31" t="str">
         <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
@@ -6538,7 +7184,7 @@
         <v>end</v>
       </c>
       <c r="C35" t="str">
-        <v>Sim</v>
+        <v>Não</v>
       </c>
       <c r="D35" t="str">
         <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
@@ -6546,547 +7192,603 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Horas Estimadas</v>
+        <v>Cronograma pelas fases</v>
       </c>
       <c r="B36" t="str">
-        <v>estimated</v>
+        <v>scheduleAuto</v>
       </c>
       <c r="C36" t="str">
         <v>Não</v>
       </c>
       <c r="D36" t="str">
-        <v>Número não negativo (ex.: 160).</v>
+        <v>Sim: datas gerais calculadas pelas fases. Não: datas manuais legadas.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Horas Consumidas</v>
+        <v>Entrega acordada com cliente</v>
       </c>
       <c r="B37" t="str">
-        <v>consumed</v>
+        <v>deadline</v>
       </c>
       <c r="C37" t="str">
         <v>Não</v>
       </c>
       <c r="D37" t="str">
-        <v>Número não negativo (ex.: 160).</v>
+        <v>Data de entrega acordada com o cliente; independente do cronograma.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Percentual de Conclusão</v>
+        <v>Horas Estimadas</v>
       </c>
       <c r="B38" t="str">
-        <v>progress</v>
+        <v>estimated</v>
       </c>
       <c r="C38" t="str">
         <v>Não</v>
       </c>
       <c r="D38" t="str">
-        <v>Percentual de 0 a 100 (ex.: 75).</v>
+        <v>Número não negativo (ex.: 160).</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Próximo Marco</v>
+        <v>Horas Consumidas</v>
       </c>
       <c r="B39" t="str">
-        <v>next</v>
+        <v>consumed</v>
       </c>
       <c r="C39" t="str">
         <v>Não</v>
       </c>
       <c r="D39" t="str">
-        <v>Texto para Próximo Marco; preserve IDs e nomes das opções.</v>
+        <v>Número não negativo (ex.: 160).</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Data Próximo Marco</v>
+        <v>Percentual de Conclusão</v>
       </c>
       <c r="B40" t="str">
-        <v>nextDate</v>
+        <v>progress</v>
       </c>
       <c r="C40" t="str">
         <v>Não</v>
       </c>
       <c r="D40" t="str">
-        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+        <v>Percentual de 0 a 100 (ex.: 75).</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Dependência</v>
+        <v>Próximo Marco</v>
       </c>
       <c r="B41" t="str">
-        <v>dependency</v>
+        <v>next</v>
       </c>
       <c r="C41" t="str">
         <v>Não</v>
       </c>
       <c r="D41" t="str">
-        <v>Texto para Dependência; preserve IDs e nomes das opções.</v>
+        <v>Texto para Próximo Marco; preserve IDs e nomes das opções.</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Responsável pela Dependência</v>
+        <v>Data Próximo Marco</v>
       </c>
       <c r="B42" t="str">
-        <v>dependencyOwner</v>
+        <v>nextDate</v>
       </c>
       <c r="C42" t="str">
         <v>Não</v>
       </c>
       <c r="D42" t="str">
-        <v>Texto para Responsável pela Dependência; preserve IDs e nomes das opções.</v>
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Risco</v>
+        <v>Dependência</v>
       </c>
       <c r="B43" t="str">
-        <v>risk</v>
+        <v>dependency</v>
       </c>
       <c r="C43" t="str">
         <v>Não</v>
       </c>
       <c r="D43" t="str">
-        <v>Use Nenhum, Baixa, Média, Alta ou Crítica.</v>
+        <v>Texto para Dependência; preserve IDs e nomes das opções.</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Descrição do Risco</v>
+        <v>Responsável pela Dependência</v>
       </c>
       <c r="B44" t="str">
-        <v>riskDescription</v>
+        <v>dependencyOwner</v>
       </c>
       <c r="C44" t="str">
         <v>Não</v>
       </c>
       <c r="D44" t="str">
-        <v>Texto para Descrição do Risco; preserve IDs e nomes das opções.</v>
+        <v>Texto para Responsável pela Dependência; preserve IDs e nomes das opções.</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Link Git</v>
+        <v>Risco</v>
       </c>
       <c r="B45" t="str">
-        <v>git</v>
+        <v>risk</v>
       </c>
       <c r="C45" t="str">
         <v>Não</v>
       </c>
       <c r="D45" t="str">
-        <v>Texto para Link Git; preserve IDs e nomes das opções.</v>
+        <v>Use Nenhum, Baixa, Média, Alta ou Crítica.</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Observação</v>
+        <v>Descrição do Risco</v>
       </c>
       <c r="B46" t="str">
-        <v>notes</v>
+        <v>riskDescription</v>
       </c>
       <c r="C46" t="str">
         <v>Não</v>
       </c>
       <c r="D46" t="str">
-        <v>Texto para Observação; preserve IDs e nomes das opções.</v>
+        <v>Texto para Descrição do Risco; preserve IDs e nomes das opções.</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
+        <v>Link Git</v>
+      </c>
+      <c r="B47" t="str">
+        <v>git</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Texto para Link Git; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Observação</v>
+      </c>
+      <c r="B48" t="str">
+        <v>notes</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Texto para Observação; preserve IDs e nomes das opções.</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
         <f>Campo</f>
         <v>Pessoas — instruções por coluna</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v>ID</v>
-      </c>
-      <c r="B48" t="str">
-        <v>id</v>
-      </c>
-      <c r="C48" t="str">
-        <v>Sim</v>
-      </c>
-      <c r="D48" t="str">
-        <v>ID único; não duplique e mantenha as referências nas outras abas.</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="str">
-        <v>Nome</v>
-      </c>
-      <c r="B49" t="str">
-        <v>name</v>
-      </c>
-      <c r="C49" t="str">
-        <v>Sim</v>
-      </c>
-      <c r="D49" t="str">
-        <v>Texto para Nome; preserve IDs e nomes das opções.</v>
-      </c>
-    </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Função</v>
+        <v>ID</v>
       </c>
       <c r="B50" t="str">
-        <v>role</v>
+        <v>id</v>
       </c>
       <c r="C50" t="str">
         <v>Sim</v>
       </c>
       <c r="D50" t="str">
-        <v>Texto para Função; preserve IDs e nomes das opções.</v>
+        <v>ID único; não duplique e mantenha as referências nas outras abas.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Frente Principal</v>
+        <v>Nome</v>
       </c>
       <c r="B51" t="str">
-        <v>front</v>
+        <v>name</v>
       </c>
       <c r="C51" t="str">
         <v>Sim</v>
       </c>
       <c r="D51" t="str">
-        <v>Use uma frente válida da lista na aba LEIA-ME.</v>
+        <v>Texto para Nome; preserve IDs e nomes das opções.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Tech Leader</v>
+        <v>Função</v>
       </c>
       <c r="B52" t="str">
-        <v>leader</v>
+        <v>role</v>
       </c>
       <c r="C52" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="D52" t="str">
-        <v>Texto para Tech Leader; preserve IDs e nomes das opções.</v>
+        <v>Texto para Função; preserve IDs e nomes das opções.</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Capacidade Mensal</v>
+        <v>Frente Principal</v>
       </c>
       <c r="B53" t="str">
-        <v>capacity</v>
+        <v>front</v>
       </c>
       <c r="C53" t="str">
         <v>Sim</v>
       </c>
       <c r="D53" t="str">
-        <v>Campo legado mantido por compatibilidade. Não altera os cálculos: a jornada é de 8h por dia, de segunda a sexta.</v>
+        <v>Use uma frente válida da lista na aba LEIA-ME.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Ativo</v>
+        <v>Tech Leader</v>
       </c>
       <c r="B54" t="str">
-        <v>active</v>
+        <v>leader</v>
       </c>
       <c r="C54" t="str">
-        <v>Sim</v>
+        <v>Não</v>
       </c>
       <c r="D54" t="str">
-        <v>Use Sim ou Não.</v>
+        <v>Texto para Tech Leader; preserve IDs e nomes das opções.</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
+        <v>Capacidade Mensal</v>
+      </c>
+      <c r="B55" t="str">
+        <v>capacity</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Campo legado mantido por compatibilidade. Não altera os cálculos: a jornada é de 8h por dia, de segunda a sexta.</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Ativo</v>
+      </c>
+      <c r="B56" t="str">
+        <v>active</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Use Sim ou Não.</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
         <f>Campo</f>
         <v>Alocacoes — instruções por coluna</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="str">
-        <v>Pessoa ID</v>
-      </c>
-      <c r="B56" t="str">
-        <v>person</v>
-      </c>
-      <c r="C56" t="str">
-        <v>Sim</v>
-      </c>
-      <c r="D56" t="str">
-        <v>ID da pessoa existente.</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="str">
-        <v>Demanda ID</v>
-      </c>
-      <c r="B57" t="str">
-        <v>demand</v>
-      </c>
-      <c r="C57" t="str">
-        <v>Sim</v>
-      </c>
-      <c r="D57" t="str">
-        <v>ID da demanda existente.</v>
-      </c>
-    </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Data Início</v>
+        <v>Pessoa ID</v>
       </c>
       <c r="B58" t="str">
-        <v>start</v>
+        <v>person</v>
       </c>
       <c r="C58" t="str">
         <v>Sim</v>
       </c>
       <c r="D58" t="str">
-        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+        <v>ID da pessoa existente.</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Data Fim</v>
+        <v>Demanda ID</v>
       </c>
       <c r="B59" t="str">
-        <v>end</v>
+        <v>demand</v>
       </c>
       <c r="C59" t="str">
         <v>Sim</v>
       </c>
       <c r="D59" t="str">
-        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+        <v>ID da demanda existente.</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Horas</v>
+        <v>Data Início</v>
       </c>
       <c r="B60" t="str">
-        <v>hours</v>
+        <v>start</v>
       </c>
       <c r="C60" t="str">
         <v>Sim</v>
       </c>
       <c r="D60" t="str">
-        <v>Horas totais do intervalo; número não negativo.</v>
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Percentual</v>
+        <v>Data Fim</v>
       </c>
       <c r="B61" t="str">
-        <v>percent</v>
+        <v>end</v>
       </c>
       <c r="C61" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="D61" t="str">
-        <v>Calculado automaticamente a partir de Horas, pessoa e período.</v>
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
+        <v>Horas</v>
+      </c>
+      <c r="B62" t="str">
+        <v>hours</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Horas totais do intervalo; número não negativo.</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>Percentual</v>
+      </c>
+      <c r="B63" t="str">
+        <v>percent</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Calculado automaticamente a partir de Horas, pessoa e período.</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
         <f>Campo</f>
         <v>Fases — instruções por coluna</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" t="str">
-        <v>Demanda ID</v>
-      </c>
-      <c r="B63" t="str">
-        <v>demand</v>
-      </c>
-      <c r="C63" t="str">
-        <v>Sim</v>
-      </c>
-      <c r="D63" t="str">
-        <v>ID da demanda existente.</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="str">
-        <v>Fase</v>
-      </c>
-      <c r="B64" t="str">
-        <v>phase</v>
-      </c>
-      <c r="C64" t="str">
-        <v>Sim</v>
-      </c>
-      <c r="D64" t="str">
-        <v>Use uma fase válida da lista na aba LEIA-ME.</v>
-      </c>
-    </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Data Início</v>
+        <v>Demanda ID</v>
       </c>
       <c r="B65" t="str">
-        <v>start</v>
+        <v>demand</v>
       </c>
       <c r="C65" t="str">
         <v>Sim</v>
       </c>
       <c r="D65" t="str">
-        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+        <v>ID da demanda existente.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Data Fim</v>
+        <v>Fase</v>
       </c>
       <c r="B66" t="str">
-        <v>end</v>
+        <v>phase</v>
       </c>
       <c r="C66" t="str">
         <v>Sim</v>
       </c>
       <c r="D66" t="str">
-        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+        <v>Use uma fase válida da lista na aba LEIA-ME.</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Status</v>
+        <v>Data Início</v>
       </c>
       <c r="B67" t="str">
-        <v>status</v>
+        <v>start</v>
       </c>
       <c r="C67" t="str">
         <v>Sim</v>
       </c>
       <c r="D67" t="str">
-        <v>Use um status válido da lista na aba LEIA-ME.</v>
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
+        <v>Data Fim</v>
+      </c>
+      <c r="B68" t="str">
+        <v>end</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>Status</v>
+      </c>
+      <c r="B69" t="str">
+        <v>status</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Use um status válido da lista na aba LEIA-ME.</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Consome horas da estimativa</v>
+      </c>
+      <c r="B70" t="str">
+        <v>budget</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Sim para reservar horas da estimativa; Não para espera sem esforço. Em arquivos antigos, vazio significa não classificado.</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Horas planejadas</v>
+      </c>
+      <c r="B71" t="str">
+        <v>plannedHours</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Horas de esforço planejadas na fase. Não são consumo realizado. Use 0 quando não consome estimativa.</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
         <f>Campo</f>
         <v>Marcos — instruções por coluna</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="str">
-        <v>Demanda ID</v>
-      </c>
-      <c r="B69" t="str">
-        <v>demand</v>
-      </c>
-      <c r="C69" t="str">
-        <v>Sim</v>
-      </c>
-      <c r="D69" t="str">
-        <v>ID da demanda existente.</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="str">
-        <v>Marco</v>
-      </c>
-      <c r="B70" t="str">
-        <v>name</v>
-      </c>
-      <c r="C70" t="str">
-        <v>Sim</v>
-      </c>
-      <c r="D70" t="str">
-        <v>Texto para Marco; preserve IDs e nomes das opções.</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="str">
-        <v>Data</v>
-      </c>
-      <c r="B71" t="str">
-        <v>date</v>
-      </c>
-      <c r="C71" t="str">
-        <v>Sim</v>
-      </c>
-      <c r="D71" t="str">
-        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="str">
-        <v>Status</v>
-      </c>
-      <c r="B72" t="str">
-        <v>status</v>
-      </c>
-      <c r="C72" t="str">
-        <v>Sim</v>
-      </c>
-      <c r="D72" t="str">
-        <v>Use um status válido da lista na aba LEIA-ME.</v>
-      </c>
-    </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Observação</v>
+        <v>Demanda ID</v>
       </c>
       <c r="B73" t="str">
-        <v>notes</v>
+        <v>demand</v>
       </c>
       <c r="C73" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="D73" t="str">
-        <v>Texto para Observação; preserve IDs e nomes das opções.</v>
+        <v>ID da demanda existente.</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Demandas — obrigatórios</v>
+        <v>Marco</v>
       </c>
       <c r="B74" t="str">
-        <v>ID; Código; Nome da Demanda; Tipo; Frente; Fase Atual; Status; Data Início; Data Final Prevista</v>
+        <v>name</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Texto para Marco; preserve IDs e nomes das opções.</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Pessoas — obrigatórios</v>
+        <v>Data</v>
       </c>
       <c r="B75" t="str">
-        <v>ID; Nome; Função; Frente Principal; Capacidade Mensal; Ativo</v>
+        <v>date</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Alocacoes — obrigatórios</v>
+        <v>Status</v>
       </c>
       <c r="B76" t="str">
-        <v>Pessoa ID; Demanda ID; Data Início; Data Fim; Horas</v>
+        <v>status</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Sim</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Use um status válido da lista na aba LEIA-ME.</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Fases — obrigatórios</v>
+        <v>Observação</v>
       </c>
       <c r="B77" t="str">
-        <v>Demanda ID; Fase; Data Início; Data Fim; Status</v>
+        <v>notes</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Não</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Texto para Observação; preserve IDs e nomes das opções.</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
+        <v>Demandas — obrigatórios</v>
+      </c>
+      <c r="B78" t="str">
+        <v>ID; Código; Nome da Demanda; Tipo; Frente; Fase Atual; Status</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Pessoas — obrigatórios</v>
+      </c>
+      <c r="B79" t="str">
+        <v>ID; Nome; Função; Frente Principal; Capacidade Mensal; Ativo</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>Alocacoes — obrigatórios</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Pessoa ID; Demanda ID; Data Início; Data Fim; Horas</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>Fases — obrigatórios</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Demanda ID; Fase; Data Início; Data Fim; Status</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
         <v>Marcos — obrigatórios</v>
       </c>
-      <c r="B78" t="str">
+      <c r="B82" t="str">
         <v>Demanda ID; Marco; Data; Status</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D78"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D82"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update demo projects for phase-based schedules and effort budgets
</commit_message>
<xml_diff>
--- a/Modelo-SGP.xlsx
+++ b/Modelo-SGP.xlsx
@@ -550,7 +550,7 @@
         <v>Melhoria Linha 1</v>
       </c>
       <c r="D2" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Produção.</v>
+        <v>Demanda demonstrativa de melhoria da operação Produção. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E2" t="str">
         <v>Melhoria</v>
@@ -586,19 +586,19 @@
         <v>2026-09-24</v>
       </c>
       <c r="P2" t="str">
-        <v>2026-09-30</v>
+        <v>2026-10-05</v>
       </c>
       <c r="Q2" t="str">
-        <v>2026-10-06</v>
+        <v>2026-10-09</v>
       </c>
       <c r="R2" t="str">
         <v>2026-10-09</v>
       </c>
       <c r="S2" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T2" t="str">
-        <v/>
+        <v>2026-10-09</v>
       </c>
       <c r="U2">
         <v>240</v>
@@ -645,7 +645,7 @@
         <v>Integração MES</v>
       </c>
       <c r="D3" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Produção.</v>
+        <v>Demanda demonstrativa de melhoria da operação Produção. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E3" t="str">
         <v>Melhoria</v>
@@ -681,19 +681,19 @@
         <v>2026-10-29</v>
       </c>
       <c r="P3" t="str">
-        <v>2026-11-04</v>
+        <v>2026-11-09</v>
       </c>
       <c r="Q3" t="str">
-        <v>2026-11-10</v>
+        <v>2026-11-13</v>
       </c>
       <c r="R3" t="str">
         <v>2026-11-13</v>
       </c>
       <c r="S3" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T3" t="str">
-        <v/>
+        <v>2026-11-13</v>
       </c>
       <c r="U3">
         <v>320</v>
@@ -740,7 +740,7 @@
         <v>Eficiência de montagem</v>
       </c>
       <c r="D4" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Produção.</v>
+        <v>Demanda demonstrativa de melhoria da operação Produção. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E4" t="str">
         <v>Proposta</v>
@@ -761,7 +761,7 @@
         <v>Business Operations</v>
       </c>
       <c r="K4" t="str">
-        <v>Proposta</v>
+        <v>Levantamento</v>
       </c>
       <c r="L4" t="str">
         <v>Não iniciado</v>
@@ -776,19 +776,19 @@
         <v>2026-12-03</v>
       </c>
       <c r="P4" t="str">
-        <v>2026-12-09</v>
+        <v>2026-12-14</v>
       </c>
       <c r="Q4" t="str">
-        <v>2026-12-15</v>
+        <v>2026-12-18</v>
       </c>
       <c r="R4" t="str">
         <v>2026-12-18</v>
       </c>
       <c r="S4" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T4" t="str">
-        <v/>
+        <v>2026-12-18</v>
       </c>
       <c r="U4">
         <v>400</v>
@@ -835,7 +835,7 @@
         <v>Rastreabilidade</v>
       </c>
       <c r="D5" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Qualidade.</v>
+        <v>Demanda demonstrativa de melhoria da operação Qualidade. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E5" t="str">
         <v>Melhoria</v>
@@ -871,19 +871,19 @@
         <v>2026-09-27</v>
       </c>
       <c r="P5" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-08</v>
       </c>
       <c r="Q5" t="str">
-        <v>2026-10-09</v>
+        <v>2026-10-12</v>
       </c>
       <c r="R5" t="str">
         <v>2026-10-12</v>
       </c>
       <c r="S5" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T5" t="str">
-        <v/>
+        <v>2026-10-12</v>
       </c>
       <c r="U5">
         <v>240</v>
@@ -930,7 +930,7 @@
         <v>Relatórios QMS</v>
       </c>
       <c r="D6" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Qualidade.</v>
+        <v>Demanda demonstrativa de melhoria da operação Qualidade. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E6" t="str">
         <v>Melhoria</v>
@@ -951,7 +951,7 @@
         <v>Business Operations</v>
       </c>
       <c r="K6" t="str">
-        <v>Aprovação</v>
+        <v>Desenvolvimento</v>
       </c>
       <c r="L6" t="str">
         <v>Aguardando aprovação</v>
@@ -966,19 +966,19 @@
         <v>2026-11-01</v>
       </c>
       <c r="P6" t="str">
-        <v>2026-11-07</v>
+        <v>2026-11-12</v>
       </c>
       <c r="Q6" t="str">
-        <v>2026-11-13</v>
+        <v>2026-11-16</v>
       </c>
       <c r="R6" t="str">
         <v>2026-11-16</v>
       </c>
       <c r="S6" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T6" t="str">
-        <v/>
+        <v>2026-11-16</v>
       </c>
       <c r="U6">
         <v>320</v>
@@ -1025,7 +1025,7 @@
         <v>Inspeção digital</v>
       </c>
       <c r="D7" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Qualidade.</v>
+        <v>Demanda demonstrativa de melhoria da operação Qualidade. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E7" t="str">
         <v>Proposta</v>
@@ -1046,7 +1046,7 @@
         <v>Business Operations</v>
       </c>
       <c r="K7" t="str">
-        <v>Proposta</v>
+        <v>Levantamento</v>
       </c>
       <c r="L7" t="str">
         <v>Não iniciado</v>
@@ -1061,19 +1061,19 @@
         <v>2026-12-06</v>
       </c>
       <c r="P7" t="str">
-        <v>2026-12-12</v>
+        <v>2026-12-17</v>
       </c>
       <c r="Q7" t="str">
-        <v>2026-12-18</v>
+        <v>2026-12-21</v>
       </c>
       <c r="R7" t="str">
         <v>2026-12-21</v>
       </c>
       <c r="S7" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T7" t="str">
-        <v/>
+        <v>2026-12-21</v>
       </c>
       <c r="U7">
         <v>400</v>
@@ -1120,7 +1120,7 @@
         <v>Calibração ERP</v>
       </c>
       <c r="D8" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Torque.</v>
+        <v>Demanda demonstrativa de melhoria da operação Torque. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E8" t="str">
         <v>Melhoria</v>
@@ -1156,19 +1156,19 @@
         <v>2026-09-30</v>
       </c>
       <c r="P8" t="str">
-        <v>2026-10-06</v>
+        <v>2026-10-11</v>
       </c>
       <c r="Q8" t="str">
-        <v>2026-10-12</v>
+        <v>2026-10-15</v>
       </c>
       <c r="R8" t="str">
         <v>2026-10-15</v>
       </c>
       <c r="S8" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T8" t="str">
-        <v/>
+        <v>2026-10-15</v>
       </c>
       <c r="U8">
         <v>240</v>
@@ -1215,7 +1215,7 @@
         <v>Coleta de Dados</v>
       </c>
       <c r="D9" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Torque.</v>
+        <v>Demanda demonstrativa de melhoria da operação Torque. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E9" t="str">
         <v>Melhoria</v>
@@ -1251,19 +1251,19 @@
         <v>2026-11-04</v>
       </c>
       <c r="P9" t="str">
-        <v>2026-11-10</v>
+        <v>2026-11-15</v>
       </c>
       <c r="Q9" t="str">
-        <v>2026-11-16</v>
+        <v>2026-11-19</v>
       </c>
       <c r="R9" t="str">
         <v>2026-11-19</v>
       </c>
       <c r="S9" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T9" t="str">
-        <v/>
+        <v>2026-11-19</v>
       </c>
       <c r="U9">
         <v>320</v>
@@ -1310,7 +1310,7 @@
         <v>Auditoria de torque</v>
       </c>
       <c r="D10" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Torque.</v>
+        <v>Demanda demonstrativa de melhoria da operação Torque. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E10" t="str">
         <v>Proposta</v>
@@ -1331,7 +1331,7 @@
         <v>Business Operations</v>
       </c>
       <c r="K10" t="str">
-        <v>Proposta</v>
+        <v>Levantamento</v>
       </c>
       <c r="L10" t="str">
         <v>Não iniciado</v>
@@ -1346,19 +1346,19 @@
         <v>2026-12-09</v>
       </c>
       <c r="P10" t="str">
-        <v>2026-12-15</v>
+        <v>2026-12-20</v>
       </c>
       <c r="Q10" t="str">
-        <v>2026-12-21</v>
+        <v>2026-12-24</v>
       </c>
       <c r="R10" t="str">
         <v>2026-12-24</v>
       </c>
       <c r="S10" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T10" t="str">
-        <v/>
+        <v>2026-12-24</v>
       </c>
       <c r="U10">
         <v>400</v>
@@ -1405,7 +1405,7 @@
         <v>Integração PLC</v>
       </c>
       <c r="D11" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Automação Industrial.</v>
+        <v>Demanda demonstrativa de melhoria da operação Automação Industrial. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E11" t="str">
         <v>Melhoria</v>
@@ -1441,19 +1441,19 @@
         <v>2026-10-03</v>
       </c>
       <c r="P11" t="str">
-        <v>2026-10-09</v>
+        <v>2026-10-14</v>
       </c>
       <c r="Q11" t="str">
-        <v>2026-10-15</v>
+        <v>2026-10-18</v>
       </c>
       <c r="R11" t="str">
         <v>2026-10-18</v>
       </c>
       <c r="S11" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T11" t="str">
-        <v/>
+        <v>2026-10-18</v>
       </c>
       <c r="U11">
         <v>240</v>
@@ -1500,7 +1500,7 @@
         <v>Dashboard IIoT</v>
       </c>
       <c r="D12" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Automação Industrial.</v>
+        <v>Demanda demonstrativa de melhoria da operação Automação Industrial. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E12" t="str">
         <v>Melhoria</v>
@@ -1536,19 +1536,19 @@
         <v>2026-11-07</v>
       </c>
       <c r="P12" t="str">
-        <v>2026-11-13</v>
+        <v>2026-11-18</v>
       </c>
       <c r="Q12" t="str">
-        <v>2026-11-19</v>
+        <v>2026-11-22</v>
       </c>
       <c r="R12" t="str">
         <v>2026-11-22</v>
       </c>
       <c r="S12" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T12" t="str">
-        <v/>
+        <v>2026-11-22</v>
       </c>
       <c r="U12">
         <v>320</v>
@@ -1595,7 +1595,7 @@
         <v>Monitoramento de células</v>
       </c>
       <c r="D13" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Automação Industrial.</v>
+        <v>Demanda demonstrativa de melhoria da operação Automação Industrial. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E13" t="str">
         <v>Proposta</v>
@@ -1616,7 +1616,7 @@
         <v>Business Operations</v>
       </c>
       <c r="K13" t="str">
-        <v>Proposta</v>
+        <v>Levantamento</v>
       </c>
       <c r="L13" t="str">
         <v>Não iniciado</v>
@@ -1631,19 +1631,19 @@
         <v>2026-12-12</v>
       </c>
       <c r="P13" t="str">
-        <v>2026-12-18</v>
+        <v>2026-12-23</v>
       </c>
       <c r="Q13" t="str">
-        <v>2026-12-24</v>
+        <v>2026-12-27</v>
       </c>
       <c r="R13" t="str">
         <v>2026-12-27</v>
       </c>
       <c r="S13" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T13" t="str">
-        <v/>
+        <v>2026-12-27</v>
       </c>
       <c r="U13">
         <v>400</v>
@@ -1690,7 +1690,7 @@
         <v>Piloto Sensor</v>
       </c>
       <c r="D14" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Inovação IoT.</v>
+        <v>Demanda demonstrativa de melhoria da operação Inovação IoT. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E14" t="str">
         <v>Melhoria</v>
@@ -1726,19 +1726,19 @@
         <v>2026-10-06</v>
       </c>
       <c r="P14" t="str">
-        <v>2026-10-12</v>
+        <v>2026-10-17</v>
       </c>
       <c r="Q14" t="str">
-        <v>2026-10-18</v>
+        <v>2026-10-21</v>
       </c>
       <c r="R14" t="str">
         <v>2026-10-21</v>
       </c>
       <c r="S14" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T14" t="str">
-        <v/>
+        <v>2026-10-21</v>
       </c>
       <c r="U14">
         <v>240</v>
@@ -1785,7 +1785,7 @@
         <v>Plataforma IoT</v>
       </c>
       <c r="D15" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Inovação IoT.</v>
+        <v>Demanda demonstrativa de melhoria da operação Inovação IoT. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E15" t="str">
         <v>Melhoria</v>
@@ -1821,19 +1821,19 @@
         <v>2026-11-10</v>
       </c>
       <c r="P15" t="str">
-        <v>2026-11-16</v>
+        <v>2026-11-21</v>
       </c>
       <c r="Q15" t="str">
-        <v>2026-11-22</v>
+        <v>2026-11-25</v>
       </c>
       <c r="R15" t="str">
         <v>2026-11-25</v>
       </c>
       <c r="S15" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T15" t="str">
-        <v/>
+        <v>2026-11-25</v>
       </c>
       <c r="U15">
         <v>320</v>
@@ -1880,7 +1880,7 @@
         <v>Conectividade industrial</v>
       </c>
       <c r="D16" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Inovação IoT.</v>
+        <v>Demanda demonstrativa de melhoria da operação Inovação IoT. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
       <c r="E16" t="str">
         <v>Proposta</v>
@@ -1901,7 +1901,7 @@
         <v>Business Operations</v>
       </c>
       <c r="K16" t="str">
-        <v>Proposta</v>
+        <v>Levantamento</v>
       </c>
       <c r="L16" t="str">
         <v>Não iniciado</v>
@@ -1916,19 +1916,19 @@
         <v>2026-12-15</v>
       </c>
       <c r="P16" t="str">
-        <v>2026-12-21</v>
+        <v>2026-12-26</v>
       </c>
       <c r="Q16" t="str">
-        <v>2026-12-27</v>
+        <v>2026-12-30</v>
       </c>
       <c r="R16" t="str">
         <v>2026-12-30</v>
       </c>
       <c r="S16" t="str">
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="T16" t="str">
-        <v/>
+        <v>2026-12-30</v>
       </c>
       <c r="U16">
         <v>400</v>
@@ -3932,13 +3932,13 @@
         <v>2026-08-27</v>
       </c>
       <c r="E2" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G2">
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -3955,13 +3955,13 @@
         <v>2026-09-01</v>
       </c>
       <c r="E3" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -3978,13 +3978,13 @@
         <v>2026-09-06</v>
       </c>
       <c r="E4" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G4">
+        <v>24</v>
       </c>
     </row>
     <row r="5">
@@ -4004,10 +4004,10 @@
         <v>Em andamento</v>
       </c>
       <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G5">
+        <v>144</v>
       </c>
     </row>
     <row r="6">
@@ -4024,13 +4024,13 @@
         <v>2026-10-05</v>
       </c>
       <c r="E6" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F6" t="str">
-        <v/>
-      </c>
-      <c r="G6" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G6">
+        <v>24</v>
       </c>
     </row>
     <row r="7">
@@ -4047,13 +4047,13 @@
         <v>2026-10-09</v>
       </c>
       <c r="E7" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F7" t="str">
-        <v/>
-      </c>
-      <c r="G7" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G7">
+        <v>24</v>
       </c>
     </row>
     <row r="8">
@@ -4070,13 +4070,13 @@
         <v>2026-09-13</v>
       </c>
       <c r="E8" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F8" t="str">
-        <v/>
-      </c>
-      <c r="G8" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G8">
+        <v>32</v>
       </c>
     </row>
     <row r="9">
@@ -4093,13 +4093,13 @@
         <v>2026-09-18</v>
       </c>
       <c r="E9" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F9" t="str">
-        <v/>
-      </c>
-      <c r="G9" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -4116,13 +4116,13 @@
         <v>2026-09-23</v>
       </c>
       <c r="E10" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F10" t="str">
-        <v/>
-      </c>
-      <c r="G10" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G10">
+        <v>32</v>
       </c>
     </row>
     <row r="11">
@@ -4142,10 +4142,10 @@
         <v>Em andamento</v>
       </c>
       <c r="F11" t="str">
-        <v/>
-      </c>
-      <c r="G11" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G11">
+        <v>192</v>
       </c>
     </row>
     <row r="12">
@@ -4162,13 +4162,13 @@
         <v>2026-11-09</v>
       </c>
       <c r="E12" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F12" t="str">
-        <v/>
-      </c>
-      <c r="G12" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G12">
+        <v>32</v>
       </c>
     </row>
     <row r="13">
@@ -4185,13 +4185,13 @@
         <v>2026-11-13</v>
       </c>
       <c r="E13" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F13" t="str">
-        <v/>
-      </c>
-      <c r="G13" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G13">
+        <v>32</v>
       </c>
     </row>
     <row r="14">
@@ -4208,13 +4208,13 @@
         <v>2026-09-30</v>
       </c>
       <c r="E14" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F14" t="str">
-        <v/>
-      </c>
-      <c r="G14" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G14">
+        <v>40</v>
       </c>
     </row>
     <row r="15">
@@ -4231,13 +4231,13 @@
         <v>2026-10-05</v>
       </c>
       <c r="E15" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F15" t="str">
-        <v/>
-      </c>
-      <c r="G15" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -4254,13 +4254,13 @@
         <v>2026-10-10</v>
       </c>
       <c r="E16" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F16" t="str">
-        <v/>
-      </c>
-      <c r="G16" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G16">
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -4277,13 +4277,13 @@
         <v>2026-12-03</v>
       </c>
       <c r="E17" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F17" t="str">
-        <v/>
-      </c>
-      <c r="G17" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G17">
+        <v>240</v>
       </c>
     </row>
     <row r="18">
@@ -4300,13 +4300,13 @@
         <v>2026-12-14</v>
       </c>
       <c r="E18" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F18" t="str">
-        <v/>
-      </c>
-      <c r="G18" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G18">
+        <v>40</v>
       </c>
     </row>
     <row r="19">
@@ -4323,13 +4323,13 @@
         <v>2026-12-18</v>
       </c>
       <c r="E19" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F19" t="str">
-        <v/>
-      </c>
-      <c r="G19" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G19">
+        <v>40</v>
       </c>
     </row>
     <row r="20">
@@ -4346,13 +4346,13 @@
         <v>2026-08-30</v>
       </c>
       <c r="E20" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F20" t="str">
-        <v/>
-      </c>
-      <c r="G20" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G20">
+        <v>24</v>
       </c>
     </row>
     <row r="21">
@@ -4369,13 +4369,13 @@
         <v>2026-09-04</v>
       </c>
       <c r="E21" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F21" t="str">
-        <v/>
-      </c>
-      <c r="G21" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -4392,13 +4392,13 @@
         <v>2026-09-09</v>
       </c>
       <c r="E22" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F22" t="str">
-        <v/>
-      </c>
-      <c r="G22" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G22">
+        <v>24</v>
       </c>
     </row>
     <row r="23">
@@ -4418,10 +4418,10 @@
         <v>Em andamento</v>
       </c>
       <c r="F23" t="str">
-        <v/>
-      </c>
-      <c r="G23" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G23">
+        <v>144</v>
       </c>
     </row>
     <row r="24">
@@ -4438,13 +4438,13 @@
         <v>2026-10-08</v>
       </c>
       <c r="E24" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F24" t="str">
-        <v/>
-      </c>
-      <c r="G24" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G24">
+        <v>24</v>
       </c>
     </row>
     <row r="25">
@@ -4461,13 +4461,13 @@
         <v>2026-10-12</v>
       </c>
       <c r="E25" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F25" t="str">
-        <v/>
-      </c>
-      <c r="G25" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G25">
+        <v>24</v>
       </c>
     </row>
     <row r="26">
@@ -4484,13 +4484,13 @@
         <v>2026-09-16</v>
       </c>
       <c r="E26" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F26" t="str">
-        <v/>
-      </c>
-      <c r="G26" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G26">
+        <v>32</v>
       </c>
     </row>
     <row r="27">
@@ -4507,13 +4507,13 @@
         <v>2026-09-21</v>
       </c>
       <c r="E27" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F27" t="str">
-        <v/>
-      </c>
-      <c r="G27" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -4530,13 +4530,13 @@
         <v>2026-09-26</v>
       </c>
       <c r="E28" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F28" t="str">
-        <v/>
-      </c>
-      <c r="G28" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G28">
+        <v>32</v>
       </c>
     </row>
     <row r="29">
@@ -4553,13 +4553,13 @@
         <v>2026-11-01</v>
       </c>
       <c r="E29" t="str">
-        <v>Em andamento</v>
+        <v>Aguardando aprovação</v>
       </c>
       <c r="F29" t="str">
-        <v/>
-      </c>
-      <c r="G29" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G29">
+        <v>192</v>
       </c>
     </row>
     <row r="30">
@@ -4576,13 +4576,13 @@
         <v>2026-11-12</v>
       </c>
       <c r="E30" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F30" t="str">
-        <v/>
-      </c>
-      <c r="G30" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G30">
+        <v>32</v>
       </c>
     </row>
     <row r="31">
@@ -4599,13 +4599,13 @@
         <v>2026-11-16</v>
       </c>
       <c r="E31" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F31" t="str">
-        <v/>
-      </c>
-      <c r="G31" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G31">
+        <v>32</v>
       </c>
     </row>
     <row r="32">
@@ -4622,13 +4622,13 @@
         <v>2026-10-03</v>
       </c>
       <c r="E32" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F32" t="str">
-        <v/>
-      </c>
-      <c r="G32" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G32">
+        <v>40</v>
       </c>
     </row>
     <row r="33">
@@ -4645,13 +4645,13 @@
         <v>2026-10-08</v>
       </c>
       <c r="E33" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F33" t="str">
-        <v/>
-      </c>
-      <c r="G33" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -4668,13 +4668,13 @@
         <v>2026-10-13</v>
       </c>
       <c r="E34" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F34" t="str">
-        <v/>
-      </c>
-      <c r="G34" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G34">
+        <v>40</v>
       </c>
     </row>
     <row r="35">
@@ -4691,13 +4691,13 @@
         <v>2026-12-06</v>
       </c>
       <c r="E35" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F35" t="str">
-        <v/>
-      </c>
-      <c r="G35" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G35">
+        <v>240</v>
       </c>
     </row>
     <row r="36">
@@ -4714,13 +4714,13 @@
         <v>2026-12-17</v>
       </c>
       <c r="E36" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F36" t="str">
-        <v/>
-      </c>
-      <c r="G36" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G36">
+        <v>40</v>
       </c>
     </row>
     <row r="37">
@@ -4737,13 +4737,13 @@
         <v>2026-12-21</v>
       </c>
       <c r="E37" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F37" t="str">
-        <v/>
-      </c>
-      <c r="G37" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G37">
+        <v>40</v>
       </c>
     </row>
     <row r="38">
@@ -4760,13 +4760,13 @@
         <v>2026-09-02</v>
       </c>
       <c r="E38" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F38" t="str">
-        <v/>
-      </c>
-      <c r="G38" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G38">
+        <v>24</v>
       </c>
     </row>
     <row r="39">
@@ -4783,13 +4783,13 @@
         <v>2026-09-07</v>
       </c>
       <c r="E39" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F39" t="str">
-        <v/>
-      </c>
-      <c r="G39" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G39">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -4806,13 +4806,13 @@
         <v>2026-09-12</v>
       </c>
       <c r="E40" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F40" t="str">
-        <v/>
-      </c>
-      <c r="G40" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G40">
+        <v>24</v>
       </c>
     </row>
     <row r="41">
@@ -4832,10 +4832,10 @@
         <v>Em andamento</v>
       </c>
       <c r="F41" t="str">
-        <v/>
-      </c>
-      <c r="G41" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G41">
+        <v>144</v>
       </c>
     </row>
     <row r="42">
@@ -4852,13 +4852,13 @@
         <v>2026-10-11</v>
       </c>
       <c r="E42" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F42" t="str">
-        <v/>
-      </c>
-      <c r="G42" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G42">
+        <v>24</v>
       </c>
     </row>
     <row r="43">
@@ -4875,13 +4875,13 @@
         <v>2026-10-15</v>
       </c>
       <c r="E43" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F43" t="str">
-        <v/>
-      </c>
-      <c r="G43" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G43">
+        <v>24</v>
       </c>
     </row>
     <row r="44">
@@ -4898,13 +4898,13 @@
         <v>2026-09-19</v>
       </c>
       <c r="E44" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F44" t="str">
-        <v/>
-      </c>
-      <c r="G44" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G44">
+        <v>32</v>
       </c>
     </row>
     <row r="45">
@@ -4921,13 +4921,13 @@
         <v>2026-09-24</v>
       </c>
       <c r="E45" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F45" t="str">
-        <v/>
-      </c>
-      <c r="G45" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G45">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -4944,13 +4944,13 @@
         <v>2026-09-29</v>
       </c>
       <c r="E46" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F46" t="str">
-        <v/>
-      </c>
-      <c r="G46" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G46">
+        <v>32</v>
       </c>
     </row>
     <row r="47">
@@ -4967,13 +4967,13 @@
         <v>2026-11-04</v>
       </c>
       <c r="E47" t="str">
-        <v>Em andamento</v>
+        <v>Aguardando cliente</v>
       </c>
       <c r="F47" t="str">
-        <v/>
-      </c>
-      <c r="G47" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G47">
+        <v>192</v>
       </c>
     </row>
     <row r="48">
@@ -4990,13 +4990,13 @@
         <v>2026-11-15</v>
       </c>
       <c r="E48" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F48" t="str">
-        <v/>
-      </c>
-      <c r="G48" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G48">
+        <v>32</v>
       </c>
     </row>
     <row r="49">
@@ -5013,13 +5013,13 @@
         <v>2026-11-19</v>
       </c>
       <c r="E49" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F49" t="str">
-        <v/>
-      </c>
-      <c r="G49" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G49">
+        <v>32</v>
       </c>
     </row>
     <row r="50">
@@ -5036,13 +5036,13 @@
         <v>2026-10-06</v>
       </c>
       <c r="E50" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F50" t="str">
-        <v/>
-      </c>
-      <c r="G50" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G50">
+        <v>40</v>
       </c>
     </row>
     <row r="51">
@@ -5059,13 +5059,13 @@
         <v>2026-10-11</v>
       </c>
       <c r="E51" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F51" t="str">
-        <v/>
-      </c>
-      <c r="G51" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G51">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -5082,13 +5082,13 @@
         <v>2026-10-16</v>
       </c>
       <c r="E52" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F52" t="str">
-        <v/>
-      </c>
-      <c r="G52" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G52">
+        <v>40</v>
       </c>
     </row>
     <row r="53">
@@ -5105,13 +5105,13 @@
         <v>2026-12-09</v>
       </c>
       <c r="E53" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F53" t="str">
-        <v/>
-      </c>
-      <c r="G53" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G53">
+        <v>240</v>
       </c>
     </row>
     <row r="54">
@@ -5128,13 +5128,13 @@
         <v>2026-12-20</v>
       </c>
       <c r="E54" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F54" t="str">
-        <v/>
-      </c>
-      <c r="G54" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G54">
+        <v>40</v>
       </c>
     </row>
     <row r="55">
@@ -5151,13 +5151,13 @@
         <v>2026-12-24</v>
       </c>
       <c r="E55" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F55" t="str">
-        <v/>
-      </c>
-      <c r="G55" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G55">
+        <v>40</v>
       </c>
     </row>
     <row r="56">
@@ -5174,13 +5174,13 @@
         <v>2026-09-05</v>
       </c>
       <c r="E56" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F56" t="str">
-        <v/>
-      </c>
-      <c r="G56" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G56">
+        <v>24</v>
       </c>
     </row>
     <row r="57">
@@ -5197,13 +5197,13 @@
         <v>2026-09-10</v>
       </c>
       <c r="E57" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F57" t="str">
-        <v/>
-      </c>
-      <c r="G57" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G57">
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -5220,13 +5220,13 @@
         <v>2026-09-15</v>
       </c>
       <c r="E58" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F58" t="str">
-        <v/>
-      </c>
-      <c r="G58" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G58">
+        <v>24</v>
       </c>
     </row>
     <row r="59">
@@ -5246,10 +5246,10 @@
         <v>Em andamento</v>
       </c>
       <c r="F59" t="str">
-        <v/>
-      </c>
-      <c r="G59" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G59">
+        <v>144</v>
       </c>
     </row>
     <row r="60">
@@ -5266,13 +5266,13 @@
         <v>2026-10-14</v>
       </c>
       <c r="E60" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F60" t="str">
-        <v/>
-      </c>
-      <c r="G60" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G60">
+        <v>24</v>
       </c>
     </row>
     <row r="61">
@@ -5289,13 +5289,13 @@
         <v>2026-10-18</v>
       </c>
       <c r="E61" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F61" t="str">
-        <v/>
-      </c>
-      <c r="G61" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G61">
+        <v>24</v>
       </c>
     </row>
     <row r="62">
@@ -5312,13 +5312,13 @@
         <v>2026-09-22</v>
       </c>
       <c r="E62" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F62" t="str">
-        <v/>
-      </c>
-      <c r="G62" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G62">
+        <v>32</v>
       </c>
     </row>
     <row r="63">
@@ -5335,13 +5335,13 @@
         <v>2026-09-27</v>
       </c>
       <c r="E63" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F63" t="str">
-        <v/>
-      </c>
-      <c r="G63" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G63">
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -5358,13 +5358,13 @@
         <v>2026-10-02</v>
       </c>
       <c r="E64" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F64" t="str">
-        <v/>
-      </c>
-      <c r="G64" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G64">
+        <v>32</v>
       </c>
     </row>
     <row r="65">
@@ -5381,13 +5381,13 @@
         <v>2026-11-07</v>
       </c>
       <c r="E65" t="str">
-        <v>Em andamento</v>
+        <v>Em risco</v>
       </c>
       <c r="F65" t="str">
-        <v/>
-      </c>
-      <c r="G65" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G65">
+        <v>192</v>
       </c>
     </row>
     <row r="66">
@@ -5404,13 +5404,13 @@
         <v>2026-11-18</v>
       </c>
       <c r="E66" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F66" t="str">
-        <v/>
-      </c>
-      <c r="G66" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G66">
+        <v>32</v>
       </c>
     </row>
     <row r="67">
@@ -5427,13 +5427,13 @@
         <v>2026-11-22</v>
       </c>
       <c r="E67" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F67" t="str">
-        <v/>
-      </c>
-      <c r="G67" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G67">
+        <v>32</v>
       </c>
     </row>
     <row r="68">
@@ -5450,13 +5450,13 @@
         <v>2026-10-09</v>
       </c>
       <c r="E68" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F68" t="str">
-        <v/>
-      </c>
-      <c r="G68" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G68">
+        <v>40</v>
       </c>
     </row>
     <row r="69">
@@ -5473,13 +5473,13 @@
         <v>2026-10-14</v>
       </c>
       <c r="E69" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F69" t="str">
-        <v/>
-      </c>
-      <c r="G69" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G69">
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -5496,13 +5496,13 @@
         <v>2026-10-19</v>
       </c>
       <c r="E70" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F70" t="str">
-        <v/>
-      </c>
-      <c r="G70" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G70">
+        <v>40</v>
       </c>
     </row>
     <row r="71">
@@ -5519,13 +5519,13 @@
         <v>2026-12-12</v>
       </c>
       <c r="E71" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F71" t="str">
-        <v/>
-      </c>
-      <c r="G71" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G71">
+        <v>240</v>
       </c>
     </row>
     <row r="72">
@@ -5542,13 +5542,13 @@
         <v>2026-12-23</v>
       </c>
       <c r="E72" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F72" t="str">
-        <v/>
-      </c>
-      <c r="G72" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G72">
+        <v>40</v>
       </c>
     </row>
     <row r="73">
@@ -5565,13 +5565,13 @@
         <v>2026-12-27</v>
       </c>
       <c r="E73" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F73" t="str">
-        <v/>
-      </c>
-      <c r="G73" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G73">
+        <v>40</v>
       </c>
     </row>
     <row r="74">
@@ -5588,13 +5588,13 @@
         <v>2026-09-08</v>
       </c>
       <c r="E74" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F74" t="str">
-        <v/>
-      </c>
-      <c r="G74" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G74">
+        <v>24</v>
       </c>
     </row>
     <row r="75">
@@ -5611,13 +5611,13 @@
         <v>2026-09-13</v>
       </c>
       <c r="E75" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F75" t="str">
-        <v/>
-      </c>
-      <c r="G75" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G75">
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -5634,13 +5634,13 @@
         <v>2026-09-18</v>
       </c>
       <c r="E76" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F76" t="str">
-        <v/>
-      </c>
-      <c r="G76" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G76">
+        <v>24</v>
       </c>
     </row>
     <row r="77">
@@ -5660,10 +5660,10 @@
         <v>Em andamento</v>
       </c>
       <c r="F77" t="str">
-        <v/>
-      </c>
-      <c r="G77" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G77">
+        <v>144</v>
       </c>
     </row>
     <row r="78">
@@ -5680,13 +5680,13 @@
         <v>2026-10-17</v>
       </c>
       <c r="E78" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F78" t="str">
-        <v/>
-      </c>
-      <c r="G78" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G78">
+        <v>24</v>
       </c>
     </row>
     <row r="79">
@@ -5703,13 +5703,13 @@
         <v>2026-10-21</v>
       </c>
       <c r="E79" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F79" t="str">
-        <v/>
-      </c>
-      <c r="G79" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G79">
+        <v>24</v>
       </c>
     </row>
     <row r="80">
@@ -5726,13 +5726,13 @@
         <v>2026-09-25</v>
       </c>
       <c r="E80" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F80" t="str">
-        <v/>
-      </c>
-      <c r="G80" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G80">
+        <v>32</v>
       </c>
     </row>
     <row r="81">
@@ -5749,13 +5749,13 @@
         <v>2026-09-30</v>
       </c>
       <c r="E81" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F81" t="str">
-        <v/>
-      </c>
-      <c r="G81" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G81">
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -5772,13 +5772,13 @@
         <v>2026-10-05</v>
       </c>
       <c r="E82" t="str">
-        <v>Em andamento</v>
+        <v>Concluído</v>
       </c>
       <c r="F82" t="str">
-        <v/>
-      </c>
-      <c r="G82" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G82">
+        <v>32</v>
       </c>
     </row>
     <row r="83">
@@ -5798,10 +5798,10 @@
         <v>Em andamento</v>
       </c>
       <c r="F83" t="str">
-        <v/>
-      </c>
-      <c r="G83" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G83">
+        <v>192</v>
       </c>
     </row>
     <row r="84">
@@ -5818,13 +5818,13 @@
         <v>2026-11-21</v>
       </c>
       <c r="E84" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F84" t="str">
-        <v/>
-      </c>
-      <c r="G84" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G84">
+        <v>32</v>
       </c>
     </row>
     <row r="85">
@@ -5841,13 +5841,13 @@
         <v>2026-11-25</v>
       </c>
       <c r="E85" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F85" t="str">
-        <v/>
-      </c>
-      <c r="G85" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G85">
+        <v>32</v>
       </c>
     </row>
     <row r="86">
@@ -5864,13 +5864,13 @@
         <v>2026-10-12</v>
       </c>
       <c r="E86" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F86" t="str">
-        <v/>
-      </c>
-      <c r="G86" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G86">
+        <v>40</v>
       </c>
     </row>
     <row r="87">
@@ -5887,13 +5887,13 @@
         <v>2026-10-17</v>
       </c>
       <c r="E87" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F87" t="str">
-        <v/>
-      </c>
-      <c r="G87" t="str">
-        <v/>
+        <v>Não</v>
+      </c>
+      <c r="G87">
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -5910,13 +5910,13 @@
         <v>2026-10-22</v>
       </c>
       <c r="E88" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F88" t="str">
-        <v/>
-      </c>
-      <c r="G88" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G88">
+        <v>40</v>
       </c>
     </row>
     <row r="89">
@@ -5933,13 +5933,13 @@
         <v>2026-12-15</v>
       </c>
       <c r="E89" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F89" t="str">
-        <v/>
-      </c>
-      <c r="G89" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G89">
+        <v>240</v>
       </c>
     </row>
     <row r="90">
@@ -5956,13 +5956,13 @@
         <v>2026-12-26</v>
       </c>
       <c r="E90" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F90" t="str">
-        <v/>
-      </c>
-      <c r="G90" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G90">
+        <v>40</v>
       </c>
     </row>
     <row r="91">
@@ -5979,13 +5979,13 @@
         <v>2026-12-30</v>
       </c>
       <c r="E91" t="str">
-        <v>Em andamento</v>
+        <v>Não iniciado</v>
       </c>
       <c r="F91" t="str">
-        <v/>
-      </c>
-      <c r="G91" t="str">
-        <v/>
+        <v>Sim</v>
+      </c>
+      <c r="G91">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Centralize demand planning in details and migrate legacy milestones
</commit_message>
<xml_diff>
--- a/Modelo-SGP.xlsx
+++ b/Modelo-SGP.xlsx
@@ -610,10 +610,10 @@
         <v>45</v>
       </c>
       <c r="X2" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y2" t="str">
-        <v>2026-09-24</v>
+        <v/>
       </c>
       <c r="Z2" t="str">
         <v/>
@@ -705,10 +705,10 @@
         <v>45</v>
       </c>
       <c r="X3" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y3" t="str">
-        <v>2026-10-29</v>
+        <v/>
       </c>
       <c r="Z3" t="str">
         <v/>
@@ -800,10 +800,10 @@
         <v>0</v>
       </c>
       <c r="X4" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y4" t="str">
-        <v>2026-12-03</v>
+        <v/>
       </c>
       <c r="Z4" t="str">
         <v/>
@@ -895,10 +895,10 @@
         <v>45</v>
       </c>
       <c r="X5" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y5" t="str">
-        <v>2026-09-27</v>
+        <v/>
       </c>
       <c r="Z5" t="str">
         <v/>
@@ -990,10 +990,10 @@
         <v>45</v>
       </c>
       <c r="X6" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y6" t="str">
-        <v>2026-11-01</v>
+        <v/>
       </c>
       <c r="Z6" t="str">
         <v>Validação do cliente</v>
@@ -1085,10 +1085,10 @@
         <v>0</v>
       </c>
       <c r="X7" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y7" t="str">
-        <v>2026-12-06</v>
+        <v/>
       </c>
       <c r="Z7" t="str">
         <v/>
@@ -1180,10 +1180,10 @@
         <v>45</v>
       </c>
       <c r="X8" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y8" t="str">
-        <v>2026-09-30</v>
+        <v/>
       </c>
       <c r="Z8" t="str">
         <v/>
@@ -1275,10 +1275,10 @@
         <v>45</v>
       </c>
       <c r="X9" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y9" t="str">
-        <v>2026-11-04</v>
+        <v/>
       </c>
       <c r="Z9" t="str">
         <v>Validação do cliente</v>
@@ -1370,10 +1370,10 @@
         <v>0</v>
       </c>
       <c r="X10" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y10" t="str">
-        <v>2026-12-09</v>
+        <v/>
       </c>
       <c r="Z10" t="str">
         <v/>
@@ -1465,10 +1465,10 @@
         <v>45</v>
       </c>
       <c r="X11" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y11" t="str">
-        <v>2026-10-03</v>
+        <v/>
       </c>
       <c r="Z11" t="str">
         <v/>
@@ -1560,10 +1560,10 @@
         <v>45</v>
       </c>
       <c r="X12" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y12" t="str">
-        <v>2026-11-07</v>
+        <v/>
       </c>
       <c r="Z12" t="str">
         <v/>
@@ -1655,10 +1655,10 @@
         <v>0</v>
       </c>
       <c r="X13" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y13" t="str">
-        <v>2026-12-12</v>
+        <v/>
       </c>
       <c r="Z13" t="str">
         <v/>
@@ -1750,10 +1750,10 @@
         <v>45</v>
       </c>
       <c r="X14" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y14" t="str">
-        <v>2026-10-06</v>
+        <v/>
       </c>
       <c r="Z14" t="str">
         <v/>
@@ -1845,10 +1845,10 @@
         <v>45</v>
       </c>
       <c r="X15" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y15" t="str">
-        <v>2026-11-10</v>
+        <v/>
       </c>
       <c r="Z15" t="str">
         <v/>
@@ -1940,10 +1940,10 @@
         <v>0</v>
       </c>
       <c r="X16" t="str">
-        <v>Entrega técnica</v>
+        <v/>
       </c>
       <c r="Y16" t="str">
-        <v>2026-12-15</v>
+        <v/>
       </c>
       <c r="Z16" t="str">
         <v/>
@@ -7271,7 +7271,7 @@
         <v>Não</v>
       </c>
       <c r="D41" t="str">
-        <v>Texto para Próximo Marco; preserve IDs e nomes das opções.</v>
+        <v>Campo legado. Cadastre os marcos na aba Marcos. Pares preenchidos serão migrados na importação.</v>
       </c>
     </row>
     <row r="42">
@@ -7285,7 +7285,7 @@
         <v>Não</v>
       </c>
       <c r="D42" t="str">
-        <v>Data em AAAA-MM-DD (ex.: 2026-09-25).</v>
+        <v>Campo legado. Use a data na aba Marcos.</v>
       </c>
     </row>
     <row r="43">

</xml_diff>

<commit_message>
Separate project summary from phase and milestone planning
</commit_message>
<xml_diff>
--- a/Modelo-SGP.xlsx
+++ b/Modelo-SGP.xlsx
@@ -550,7 +550,7 @@
         <v>Melhoria Linha 1</v>
       </c>
       <c r="D2" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Produção. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Produção.</v>
       </c>
       <c r="E2" t="str">
         <v>Melhoria</v>
@@ -631,7 +631,7 @@
         <v/>
       </c>
       <c r="AE2" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
     <row r="3">
@@ -645,7 +645,7 @@
         <v>Integração MES</v>
       </c>
       <c r="D3" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Produção. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Produção.</v>
       </c>
       <c r="E3" t="str">
         <v>Melhoria</v>
@@ -726,7 +726,7 @@
         <v/>
       </c>
       <c r="AE3" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
     <row r="4">
@@ -740,7 +740,7 @@
         <v>Eficiência de montagem</v>
       </c>
       <c r="D4" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Produção. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Produção.</v>
       </c>
       <c r="E4" t="str">
         <v>Proposta</v>
@@ -821,7 +821,7 @@
         <v/>
       </c>
       <c r="AE4" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
     <row r="5">
@@ -835,7 +835,7 @@
         <v>Rastreabilidade</v>
       </c>
       <c r="D5" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Qualidade. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Qualidade.</v>
       </c>
       <c r="E5" t="str">
         <v>Melhoria</v>
@@ -916,7 +916,7 @@
         <v/>
       </c>
       <c r="AE5" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
     <row r="6">
@@ -930,7 +930,7 @@
         <v>Relatórios QMS</v>
       </c>
       <c r="D6" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Qualidade. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Qualidade.</v>
       </c>
       <c r="E6" t="str">
         <v>Melhoria</v>
@@ -1011,7 +1011,7 @@
         <v/>
       </c>
       <c r="AE6" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
     <row r="7">
@@ -1025,7 +1025,7 @@
         <v>Inspeção digital</v>
       </c>
       <c r="D7" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Qualidade. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Qualidade.</v>
       </c>
       <c r="E7" t="str">
         <v>Proposta</v>
@@ -1106,7 +1106,7 @@
         <v/>
       </c>
       <c r="AE7" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
     <row r="8">
@@ -1120,7 +1120,7 @@
         <v>Calibração ERP</v>
       </c>
       <c r="D8" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Torque. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Torque.</v>
       </c>
       <c r="E8" t="str">
         <v>Melhoria</v>
@@ -1201,7 +1201,7 @@
         <v/>
       </c>
       <c r="AE8" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
     <row r="9">
@@ -1215,7 +1215,7 @@
         <v>Coleta de Dados</v>
       </c>
       <c r="D9" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Torque. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Torque.</v>
       </c>
       <c r="E9" t="str">
         <v>Melhoria</v>
@@ -1296,7 +1296,7 @@
         <v/>
       </c>
       <c r="AE9" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
     <row r="10">
@@ -1310,7 +1310,7 @@
         <v>Auditoria de torque</v>
       </c>
       <c r="D10" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Torque. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Torque.</v>
       </c>
       <c r="E10" t="str">
         <v>Proposta</v>
@@ -1391,7 +1391,7 @@
         <v/>
       </c>
       <c r="AE10" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
     <row r="11">
@@ -1405,7 +1405,7 @@
         <v>Integração PLC</v>
       </c>
       <c r="D11" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Automação Industrial. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Automação Industrial.</v>
       </c>
       <c r="E11" t="str">
         <v>Melhoria</v>
@@ -1486,7 +1486,7 @@
         <v/>
       </c>
       <c r="AE11" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
     <row r="12">
@@ -1500,7 +1500,7 @@
         <v>Dashboard IIoT</v>
       </c>
       <c r="D12" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Automação Industrial. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Automação Industrial.</v>
       </c>
       <c r="E12" t="str">
         <v>Melhoria</v>
@@ -1581,7 +1581,7 @@
         <v/>
       </c>
       <c r="AE12" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
     <row r="13">
@@ -1595,7 +1595,7 @@
         <v>Monitoramento de células</v>
       </c>
       <c r="D13" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Automação Industrial. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Automação Industrial.</v>
       </c>
       <c r="E13" t="str">
         <v>Proposta</v>
@@ -1676,7 +1676,7 @@
         <v/>
       </c>
       <c r="AE13" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
     <row r="14">
@@ -1690,7 +1690,7 @@
         <v>Piloto Sensor</v>
       </c>
       <c r="D14" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Inovação IoT. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Inovação IoT.</v>
       </c>
       <c r="E14" t="str">
         <v>Melhoria</v>
@@ -1771,7 +1771,7 @@
         <v/>
       </c>
       <c r="AE14" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
     <row r="15">
@@ -1785,7 +1785,7 @@
         <v>Plataforma IoT</v>
       </c>
       <c r="D15" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Inovação IoT. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Inovação IoT.</v>
       </c>
       <c r="E15" t="str">
         <v>Melhoria</v>
@@ -1866,7 +1866,7 @@
         <v/>
       </c>
       <c r="AE15" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
     <row r="16">
@@ -1880,7 +1880,7 @@
         <v>Conectividade industrial</v>
       </c>
       <c r="D16" t="str">
-        <v>Demanda demonstrativa de melhoria da operação Inovação IoT. Fases com esforço reservado; Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
+        <v>Demanda demonstrativa de melhoria da operação Inovação IoT.</v>
       </c>
       <c r="E16" t="str">
         <v>Proposta</v>
@@ -1961,7 +1961,7 @@
         <v/>
       </c>
       <c r="AE16" t="str">
-        <v>Dados fictícios para demonstração.</v>
+        <v>Exemplo com fases, marcos e alocações separados. Proposta representa espera pela decisão do cliente, sem consumo de horas.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add SGP-Global demand type and global filter
</commit_message>
<xml_diff>
--- a/Modelo-SGP.xlsx
+++ b/Modelo-SGP.xlsx
@@ -6889,7 +6889,7 @@
         <v>Tipo</v>
       </c>
       <c r="B11" t="str">
-        <v>Projeto; Proposta; Melhoria; Evolução; Ticket N3; Outro</v>
+        <v>Projeto; Proposta; Melhoria; Evolução; Ticket N3; SGP-Global; Outro</v>
       </c>
     </row>
     <row r="12">
@@ -7005,7 +7005,7 @@
         <v>Sim</v>
       </c>
       <c r="D22" t="str">
-        <v>Use Projeto, Proposta, Melhoria, Evolução, Ticket N3 ou Outro.</v>
+        <v>Use uma das opções de Tipo na aba LEIA-ME, incluindo SGP-Global.</v>
       </c>
     </row>
     <row r="23">

</xml_diff>